<commit_message>
Regenerate workbook with highlighted minus signs on negatives
Discriminativo now shows contractionary flows with a typographic minus,
bold red type, and red fill instead of parentheses.

Co-authored-by: cafla19791 <cafla19791@gmail.com>
</commit_message>
<xml_diff>
--- a/output/fatores_condicionantes_base_monetaria.xlsx
+++ b/output/fatores_condicionantes_base_monetaria.xlsx
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.0;(#,##0.0);&quot;—&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0.0;&quot;−&quot;#,##0.0;&quot;—&quot;"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -68,7 +68,8 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="009C0006"/>
+      <b val="1"/>
+      <color rgb="009B1B1B"/>
       <sz val="9"/>
     </font>
     <font>
@@ -111,7 +112,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -125,7 +126,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -136,6 +137,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -202,16 +208,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -220,30 +226,30 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -255,10 +261,10 @@
     <xf numFmtId="164" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="12" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="12" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -954,7 +960,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>30/08/2026 15:09</t>
+          <t>30/08/2026 16:01</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1164,7 @@
     <row r="2" ht="36" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Cada linha é um ano. As colunas dos fatores são o fluxo acumulado no ano (R$ milhões). A coluna «Variação da base monetária» é a soma algébrica dos oito fatores (fórmula SOMA; primário e secundário são detalhe do total de títulos e não entram de novo). 2026* = até o último mês publicado.</t>
+          <t>Cada linha é um ano. As colunas dos fatores são o fluxo acumulado no ano (R$ milhões). A coluna «Variação da base monetária» é a soma algébrica dos oito fatores (fórmula SOMA; primário e secundário são detalhe do total de títulos e não entram de novo). 2026* = até o último mês publicado. Valores negativos: sinal − em vermelho negrito, com fundo vermelho.</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1275,7 @@
       <c r="I5" s="8" t="n">
         <v>-839.2619999999999</v>
       </c>
-      <c r="J5" s="11">
+      <c r="J5" s="8">
         <f>SUM(B5:I5)</f>
         <v/>
       </c>
@@ -1279,18 +1285,18 @@
       <c r="L5" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="M5" s="11" t="n">
         <v>47686.213</v>
       </c>
-      <c r="N5" s="12" t="n">
+      <c r="N5" s="11" t="n">
         <v>32633.056</v>
       </c>
-      <c r="O5" s="12" t="n">
+      <c r="O5" s="11" t="n">
         <v>15053.157</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>2001</t>
         </is>
@@ -1319,7 +1325,7 @@
       <c r="I6" s="8" t="n">
         <v>-3424.281</v>
       </c>
-      <c r="J6" s="11">
+      <c r="J6" s="13">
         <f>SUM(B6:I6)</f>
         <v/>
       </c>
@@ -1329,13 +1335,13 @@
       <c r="L6" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="M6" s="11" t="n">
         <v>53255.971</v>
       </c>
-      <c r="N6" s="12" t="n">
+      <c r="N6" s="11" t="n">
         <v>37668.836</v>
       </c>
-      <c r="O6" s="12" t="n">
+      <c r="O6" s="11" t="n">
         <v>15587.135</v>
       </c>
     </row>
@@ -1369,7 +1375,7 @@
       <c r="I7" s="8" t="n">
         <v>-1338.211</v>
       </c>
-      <c r="J7" s="11">
+      <c r="J7" s="13">
         <f>SUM(B7:I7)</f>
         <v/>
       </c>
@@ -1379,18 +1385,18 @@
       <c r="L7" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M7" s="12" t="n">
+      <c r="M7" s="11" t="n">
         <v>73302.272</v>
       </c>
-      <c r="N7" s="12" t="n">
+      <c r="N7" s="11" t="n">
         <v>49931.066</v>
       </c>
-      <c r="O7" s="12" t="n">
+      <c r="O7" s="11" t="n">
         <v>23371.206</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>2003</t>
         </is>
@@ -1419,7 +1425,7 @@
       <c r="I8" s="8" t="n">
         <v>-1941.998</v>
       </c>
-      <c r="J8" s="11">
+      <c r="J8" s="8">
         <f>SUM(B8:I8)</f>
         <v/>
       </c>
@@ -1429,13 +1435,13 @@
       <c r="L8" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M8" s="12" t="n">
+      <c r="M8" s="11" t="n">
         <v>73219.136</v>
       </c>
-      <c r="N8" s="12" t="n">
+      <c r="N8" s="11" t="n">
         <v>51363.863</v>
       </c>
-      <c r="O8" s="12" t="n">
+      <c r="O8" s="11" t="n">
         <v>21855.273</v>
       </c>
     </row>
@@ -1469,7 +1475,7 @@
       <c r="I9" s="8" t="n">
         <v>-148.935</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="13">
         <f>SUM(B9:I9)</f>
         <v/>
       </c>
@@ -1479,18 +1485,18 @@
       <c r="L9" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="M9" s="11" t="n">
         <v>88732.677</v>
       </c>
-      <c r="N9" s="12" t="n">
+      <c r="N9" s="11" t="n">
         <v>61935.635</v>
       </c>
-      <c r="O9" s="12" t="n">
+      <c r="O9" s="11" t="n">
         <v>26797.042</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>2005</t>
         </is>
@@ -1519,7 +1525,7 @@
       <c r="I10" s="9" t="n">
         <v>632.9059999999999</v>
       </c>
-      <c r="J10" s="11">
+      <c r="J10" s="13">
         <f>SUM(B10:I10)</f>
         <v/>
       </c>
@@ -1529,13 +1535,13 @@
       <c r="L10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="M10" s="11" t="n">
         <v>101247.235</v>
       </c>
-      <c r="N10" s="12" t="n">
+      <c r="N10" s="11" t="n">
         <v>70033.641</v>
       </c>
-      <c r="O10" s="12" t="n">
+      <c r="O10" s="11" t="n">
         <v>31213.594</v>
       </c>
     </row>
@@ -1569,7 +1575,7 @@
       <c r="I11" s="9" t="n">
         <v>1012.499</v>
       </c>
-      <c r="J11" s="11">
+      <c r="J11" s="13">
         <f>SUM(B11:I11)</f>
         <v/>
       </c>
@@ -1579,18 +1585,18 @@
       <c r="L11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="M11" s="11" t="n">
         <v>121102.001</v>
       </c>
-      <c r="N11" s="12" t="n">
+      <c r="N11" s="11" t="n">
         <v>85824.753</v>
       </c>
-      <c r="O11" s="12" t="n">
+      <c r="O11" s="11" t="n">
         <v>35277.248</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>2007</t>
         </is>
@@ -1619,7 +1625,7 @@
       <c r="I12" s="9" t="n">
         <v>1491.448</v>
       </c>
-      <c r="J12" s="11">
+      <c r="J12" s="13">
         <f>SUM(B12:I12)</f>
         <v/>
       </c>
@@ -1629,13 +1635,13 @@
       <c r="L12" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="M12" s="11" t="n">
         <v>146616.867</v>
       </c>
-      <c r="N12" s="12" t="n">
+      <c r="N12" s="11" t="n">
         <v>102885.047</v>
       </c>
-      <c r="O12" s="12" t="n">
+      <c r="O12" s="11" t="n">
         <v>43731.82</v>
       </c>
     </row>
@@ -1669,7 +1675,7 @@
       <c r="I13" s="9" t="n">
         <v>1071.994</v>
       </c>
-      <c r="J13" s="11">
+      <c r="J13" s="13">
         <f>SUM(B13:I13)</f>
         <v/>
       </c>
@@ -1679,18 +1685,18 @@
       <c r="L13" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M13" s="12" t="n">
+      <c r="M13" s="11" t="n">
         <v>147549.705</v>
       </c>
-      <c r="N13" s="12" t="n">
+      <c r="N13" s="11" t="n">
         <v>115590.704</v>
       </c>
-      <c r="O13" s="12" t="n">
+      <c r="O13" s="11" t="n">
         <v>31959.001</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>2009</t>
         </is>
@@ -1719,7 +1725,7 @@
       <c r="I14" s="9" t="n">
         <v>3242.878</v>
       </c>
-      <c r="J14" s="11">
+      <c r="J14" s="13">
         <f>SUM(B14:I14)</f>
         <v/>
       </c>
@@ -1729,13 +1735,13 @@
       <c r="L14" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M14" s="12" t="n">
+      <c r="M14" s="11" t="n">
         <v>166072.835</v>
       </c>
-      <c r="N14" s="12" t="n">
+      <c r="N14" s="11" t="n">
         <v>131861.185</v>
       </c>
-      <c r="O14" s="12" t="n">
+      <c r="O14" s="11" t="n">
         <v>34211.65</v>
       </c>
     </row>
@@ -1769,7 +1775,7 @@
       <c r="I15" s="9" t="n">
         <v>3829.68</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J15" s="13">
         <f>SUM(B15:I15)</f>
         <v/>
       </c>
@@ -1779,18 +1785,18 @@
       <c r="L15" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="M15" s="11" t="n">
         <v>206853.322</v>
       </c>
-      <c r="N15" s="12" t="n">
+      <c r="N15" s="11" t="n">
         <v>151145.368</v>
       </c>
-      <c r="O15" s="12" t="n">
+      <c r="O15" s="11" t="n">
         <v>55707.954</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>2011</t>
         </is>
@@ -1819,7 +1825,7 @@
       <c r="I16" s="9" t="n">
         <v>2756.678</v>
       </c>
-      <c r="J16" s="11">
+      <c r="J16" s="13">
         <f>SUM(B16:I16)</f>
         <v/>
       </c>
@@ -1829,13 +1835,13 @@
       <c r="L16" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="M16" s="11" t="n">
         <v>214235.311</v>
       </c>
-      <c r="N16" s="12" t="n">
+      <c r="N16" s="11" t="n">
         <v>162769.67</v>
       </c>
-      <c r="O16" s="12" t="n">
+      <c r="O16" s="11" t="n">
         <v>51465.641</v>
       </c>
     </row>
@@ -1869,7 +1875,7 @@
       <c r="I17" s="8" t="n">
         <v>-8392.875</v>
       </c>
-      <c r="J17" s="11">
+      <c r="J17" s="13">
         <f>SUM(B17:I17)</f>
         <v/>
       </c>
@@ -1879,18 +1885,18 @@
       <c r="L17" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="M17" s="11" t="n">
         <v>233371.452</v>
       </c>
-      <c r="N17" s="12" t="n">
+      <c r="N17" s="11" t="n">
         <v>187434.736</v>
       </c>
-      <c r="O17" s="12" t="n">
+      <c r="O17" s="11" t="n">
         <v>45936.716</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>2013</t>
         </is>
@@ -1919,7 +1925,7 @@
       <c r="I18" s="8" t="n">
         <v>-12532.941</v>
       </c>
-      <c r="J18" s="11">
+      <c r="J18" s="13">
         <f>SUM(B18:I18)</f>
         <v/>
       </c>
@@ -1929,13 +1935,13 @@
       <c r="L18" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="M18" s="11" t="n">
         <v>249509.778</v>
       </c>
-      <c r="N18" s="12" t="n">
+      <c r="N18" s="11" t="n">
         <v>204052.42</v>
       </c>
-      <c r="O18" s="12" t="n">
+      <c r="O18" s="11" t="n">
         <v>45457.358</v>
       </c>
     </row>
@@ -1969,7 +1975,7 @@
       <c r="I19" s="9" t="n">
         <v>1227.406</v>
       </c>
-      <c r="J19" s="11">
+      <c r="J19" s="13">
         <f>SUM(B19:I19)</f>
         <v/>
       </c>
@@ -1979,18 +1985,18 @@
       <c r="L19" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="M19" s="12" t="n">
+      <c r="M19" s="11" t="n">
         <v>263528.517</v>
       </c>
-      <c r="N19" s="12" t="n">
+      <c r="N19" s="11" t="n">
         <v>220853.706</v>
       </c>
-      <c r="O19" s="12" t="n">
+      <c r="O19" s="11" t="n">
         <v>42674.811</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>2015</t>
         </is>
@@ -2019,7 +2025,7 @@
       <c r="I20" s="9" t="n">
         <v>6233.098</v>
       </c>
-      <c r="J20" s="11">
+      <c r="J20" s="8">
         <f>SUM(B20:I20)</f>
         <v/>
       </c>
@@ -2029,13 +2035,13 @@
       <c r="L20" s="8" t="n">
         <v>-536.6</v>
       </c>
-      <c r="M20" s="12" t="n">
+      <c r="M20" s="11" t="n">
         <v>255288.922</v>
       </c>
-      <c r="N20" s="12" t="n">
+      <c r="N20" s="11" t="n">
         <v>225485.184</v>
       </c>
-      <c r="O20" s="12" t="n">
+      <c r="O20" s="11" t="n">
         <v>29803.738</v>
       </c>
     </row>
@@ -2069,7 +2075,7 @@
       <c r="I21" s="9" t="n">
         <v>7424.617</v>
       </c>
-      <c r="J21" s="11">
+      <c r="J21" s="13">
         <f>SUM(B21:I21)</f>
         <v/>
       </c>
@@ -2079,18 +2085,18 @@
       <c r="L21" s="9" t="n">
         <v>370.936</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="M21" s="11" t="n">
         <v>270287.146</v>
       </c>
-      <c r="N21" s="12" t="n">
+      <c r="N21" s="11" t="n">
         <v>232145.593</v>
       </c>
-      <c r="O21" s="12" t="n">
+      <c r="O21" s="11" t="n">
         <v>38141.553</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>2017</t>
         </is>
@@ -2119,7 +2125,7 @@
       <c r="I22" s="9" t="n">
         <v>5896.818</v>
       </c>
-      <c r="J22" s="11">
+      <c r="J22" s="13">
         <f>SUM(B22:I22)</f>
         <v/>
       </c>
@@ -2129,13 +2135,13 @@
       <c r="L22" s="9" t="n">
         <v>84375.56600000001</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="M22" s="11" t="n">
         <v>296755.456</v>
       </c>
-      <c r="N22" s="12" t="n">
+      <c r="N22" s="11" t="n">
         <v>250363.681</v>
       </c>
-      <c r="O22" s="12" t="n">
+      <c r="O22" s="11" t="n">
         <v>46391.775</v>
       </c>
     </row>
@@ -2169,7 +2175,7 @@
       <c r="I23" s="9" t="n">
         <v>2909.758</v>
       </c>
-      <c r="J23" s="11">
+      <c r="J23" s="13">
         <f>SUM(B23:I23)</f>
         <v/>
       </c>
@@ -2179,18 +2185,18 @@
       <c r="L23" s="9" t="n">
         <v>2389.234</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="M23" s="11" t="n">
         <v>302049.461</v>
       </c>
-      <c r="N23" s="12" t="n">
+      <c r="N23" s="11" t="n">
         <v>264967.669</v>
       </c>
-      <c r="O23" s="12" t="n">
+      <c r="O23" s="11" t="n">
         <v>37081.792</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
@@ -2219,7 +2225,7 @@
       <c r="I24" s="8" t="n">
         <v>-6634.019</v>
       </c>
-      <c r="J24" s="11">
+      <c r="J24" s="13">
         <f>SUM(B24:I24)</f>
         <v/>
       </c>
@@ -2229,13 +2235,13 @@
       <c r="L24" s="9" t="n">
         <v>243045.615</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="M24" s="11" t="n">
         <v>316586.707</v>
       </c>
-      <c r="N24" s="12" t="n">
+      <c r="N24" s="11" t="n">
         <v>280685.185</v>
       </c>
-      <c r="O24" s="12" t="n">
+      <c r="O24" s="11" t="n">
         <v>35901.522</v>
       </c>
     </row>
@@ -2269,7 +2275,7 @@
       <c r="I25" s="8" t="n">
         <v>-19343.055</v>
       </c>
-      <c r="J25" s="11">
+      <c r="J25" s="13">
         <f>SUM(B25:I25)</f>
         <v/>
       </c>
@@ -2279,18 +2285,18 @@
       <c r="L25" s="8" t="n">
         <v>-264574.325</v>
       </c>
-      <c r="M25" s="12" t="n">
+      <c r="M25" s="11" t="n">
         <v>431536.653</v>
       </c>
-      <c r="N25" s="12" t="n">
+      <c r="N25" s="11" t="n">
         <v>370441.036</v>
       </c>
-      <c r="O25" s="12" t="n">
+      <c r="O25" s="11" t="n">
         <v>61095.617</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>2021</t>
         </is>
@@ -2319,7 +2325,7 @@
       <c r="I26" s="8" t="n">
         <v>-30402.627</v>
       </c>
-      <c r="J26" s="11">
+      <c r="J26" s="8">
         <f>SUM(B26:I26)</f>
         <v/>
       </c>
@@ -2329,13 +2335,13 @@
       <c r="L26" s="9" t="n">
         <v>303982.035</v>
       </c>
-      <c r="M26" s="12" t="n">
+      <c r="M26" s="11" t="n">
         <v>409183.519</v>
       </c>
-      <c r="N26" s="12" t="n">
+      <c r="N26" s="11" t="n">
         <v>339013.043</v>
       </c>
-      <c r="O26" s="12" t="n">
+      <c r="O26" s="11" t="n">
         <v>70170.476</v>
       </c>
     </row>
@@ -2369,7 +2375,7 @@
       <c r="I27" s="8" t="n">
         <v>-80194.454</v>
       </c>
-      <c r="J27" s="11">
+      <c r="J27" s="13">
         <f>SUM(B27:I27)</f>
         <v/>
       </c>
@@ -2379,18 +2385,18 @@
       <c r="L27" s="9" t="n">
         <v>185991.949</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="M27" s="11" t="n">
         <v>419659.918</v>
       </c>
-      <c r="N27" s="12" t="n">
+      <c r="N27" s="11" t="n">
         <v>342334.138</v>
       </c>
-      <c r="O27" s="12" t="n">
+      <c r="O27" s="11" t="n">
         <v>77325.78</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>2023</t>
         </is>
@@ -2419,7 +2425,7 @@
       <c r="I28" s="8" t="n">
         <v>-75435.61500000001</v>
       </c>
-      <c r="J28" s="11">
+      <c r="J28" s="13">
         <f>SUM(B28:I28)</f>
         <v/>
       </c>
@@ -2429,13 +2435,13 @@
       <c r="L28" s="8" t="n">
         <v>-130320.548</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="M28" s="11" t="n">
         <v>422718.628</v>
       </c>
-      <c r="N28" s="12" t="n">
+      <c r="N28" s="11" t="n">
         <v>341616.828</v>
       </c>
-      <c r="O28" s="12" t="n">
+      <c r="O28" s="11" t="n">
         <v>81101.8</v>
       </c>
     </row>
@@ -2469,7 +2475,7 @@
       <c r="I29" s="8" t="n">
         <v>-98786.795</v>
       </c>
-      <c r="J29" s="11">
+      <c r="J29" s="13">
         <f>SUM(B29:I29)</f>
         <v/>
       </c>
@@ -2479,18 +2485,18 @@
       <c r="L29" s="9" t="n">
         <v>93569.787</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="M29" s="11" t="n">
         <v>451213.588</v>
       </c>
-      <c r="N29" s="12" t="n">
+      <c r="N29" s="11" t="n">
         <v>355858.101</v>
       </c>
-      <c r="O29" s="12" t="n">
+      <c r="O29" s="11" t="n">
         <v>95355.488</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="12" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
@@ -2519,7 +2525,7 @@
       <c r="I30" s="8" t="n">
         <v>-100762.164</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30" s="8">
         <f>SUM(B30:I30)</f>
         <v/>
       </c>
@@ -2529,13 +2535,13 @@
       <c r="L30" s="9" t="n">
         <v>430597.121</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="M30" s="11" t="n">
         <v>447096.654</v>
       </c>
-      <c r="N30" s="12" t="n">
+      <c r="N30" s="11" t="n">
         <v>368625.466</v>
       </c>
-      <c r="O30" s="12" t="n">
+      <c r="O30" s="11" t="n">
         <v>78471.18799999999</v>
       </c>
     </row>
@@ -2569,7 +2575,7 @@
       <c r="I31" s="8" t="n">
         <v>-133484.659</v>
       </c>
-      <c r="J31" s="11">
+      <c r="J31" s="8">
         <f>SUM(B31:I31)</f>
         <v/>
       </c>
@@ -2579,13 +2585,13 @@
       <c r="L31" s="8" t="n">
         <v>-199640.393</v>
       </c>
-      <c r="M31" s="12" t="n">
+      <c r="M31" s="11" t="n">
         <v>432551.687</v>
       </c>
-      <c r="N31" s="12" t="n">
+      <c r="N31" s="11" t="n">
         <v>382994.849</v>
       </c>
-      <c r="O31" s="12" t="n">
+      <c r="O31" s="11" t="n">
         <v>49556.839</v>
       </c>
     </row>
@@ -2595,39 +2601,39 @@
           <t>Total fluxos</t>
         </is>
       </c>
-      <c r="B32" s="11">
+      <c r="B32" s="13">
         <f>SUM(B5:B31)</f>
         <v/>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="13">
         <f>SUM(C5:C31)</f>
         <v/>
       </c>
-      <c r="D32" s="11">
+      <c r="D32" s="13">
         <f>SUM(D5:D31)</f>
         <v/>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="13">
         <f>SUM(E5:E31)</f>
         <v/>
       </c>
-      <c r="F32" s="11">
+      <c r="F32" s="13">
         <f>SUM(F5:F31)</f>
         <v/>
       </c>
-      <c r="G32" s="11">
+      <c r="G32" s="13">
         <f>SUM(G5:G31)</f>
         <v/>
       </c>
-      <c r="H32" s="11">
+      <c r="H32" s="13">
         <f>SUM(H5:H31)</f>
         <v/>
       </c>
-      <c r="I32" s="11">
+      <c r="I32" s="13">
         <f>SUM(I5:I31)</f>
         <v/>
       </c>
-      <c r="J32" s="11">
+      <c r="J32" s="13">
         <f>SUM(J5:J31)</f>
         <v/>
       </c>
@@ -2640,7 +2646,7 @@
     <row r="34">
       <c r="A34" s="16" t="inlineStr">
         <is>
-          <t>Valores em R$ milhões. Verde = expansão; vermelho = contração. «Variação da base monetária» = SOMA algébrica das oito colunas de fatores da mesma linha.</t>
+          <t>Valores em R$ milhões. Verde = expansão; vermelho = contração. «Variação da base monetária» = SOMA algébrica das oito colunas de fatores da mesma linha. Negativos: sinal − vermelho negrito sobre fundo vermelho.</t>
         </is>
       </c>
     </row>
@@ -2867,85 +2873,85 @@
           <t>1810</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="8" t="n">
         <v>-26539.148</v>
       </c>
-      <c r="D5" s="20" t="n">
+      <c r="D5" s="8" t="n">
         <v>-11944.926</v>
       </c>
-      <c r="E5" s="20" t="n">
+      <c r="E5" s="8" t="n">
         <v>-20483.697</v>
       </c>
-      <c r="F5" s="20" t="n">
+      <c r="F5" s="8" t="n">
         <v>-1064.493</v>
       </c>
-      <c r="G5" s="20" t="n">
+      <c r="G5" s="8" t="n">
         <v>-48292.47</v>
       </c>
-      <c r="H5" s="20" t="n">
+      <c r="H5" s="8" t="n">
         <v>-43007.731</v>
       </c>
-      <c r="I5" s="20" t="n">
+      <c r="I5" s="8" t="n">
         <v>-59510.709</v>
       </c>
-      <c r="J5" s="20" t="n">
+      <c r="J5" s="8" t="n">
         <v>-55600.882</v>
       </c>
-      <c r="K5" s="20" t="n">
+      <c r="K5" s="8" t="n">
         <v>-74312.39599999999</v>
       </c>
-      <c r="L5" s="20" t="n">
+      <c r="L5" s="8" t="n">
         <v>-52311.507</v>
       </c>
-      <c r="M5" s="20" t="n">
+      <c r="M5" s="8" t="n">
         <v>-51203.673</v>
       </c>
-      <c r="N5" s="20" t="n">
+      <c r="N5" s="8" t="n">
         <v>-125632.863</v>
       </c>
-      <c r="O5" s="20" t="n">
+      <c r="O5" s="8" t="n">
         <v>-121648.972</v>
       </c>
-      <c r="P5" s="20" t="n">
+      <c r="P5" s="8" t="n">
         <v>-127554.789</v>
       </c>
-      <c r="Q5" s="20" t="n">
+      <c r="Q5" s="8" t="n">
         <v>-668.486</v>
       </c>
-      <c r="R5" s="21" t="n">
+      <c r="R5" s="20" t="n">
         <v>59665.808</v>
       </c>
-      <c r="S5" s="21" t="n">
+      <c r="S5" s="20" t="n">
         <v>12284.191</v>
       </c>
-      <c r="T5" s="21" t="n">
+      <c r="T5" s="20" t="n">
         <v>52132.877</v>
       </c>
-      <c r="U5" s="20" t="n">
+      <c r="U5" s="8" t="n">
         <v>-44486.13</v>
       </c>
-      <c r="V5" s="20" t="n">
+      <c r="V5" s="8" t="n">
         <v>-89301.052</v>
       </c>
-      <c r="W5" s="21" t="n">
+      <c r="W5" s="20" t="n">
         <v>704194.5379999999</v>
       </c>
-      <c r="X5" s="20" t="n">
+      <c r="X5" s="8" t="n">
         <v>-81290.481</v>
       </c>
-      <c r="Y5" s="20" t="n">
+      <c r="Y5" s="8" t="n">
         <v>-152518.591</v>
       </c>
-      <c r="Z5" s="21" t="n">
+      <c r="Z5" s="20" t="n">
         <v>206854.972</v>
       </c>
-      <c r="AA5" s="21" t="n">
+      <c r="AA5" s="20" t="n">
         <v>65831.935</v>
       </c>
-      <c r="AB5" s="21" t="n">
+      <c r="AB5" s="20" t="n">
         <v>94770.505</v>
       </c>
-      <c r="AC5" s="21" t="n">
+      <c r="AC5" s="20" t="n">
         <v>174826.19</v>
       </c>
     </row>
@@ -2960,85 +2966,85 @@
           <t>1811</t>
         </is>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="20" t="n">
         <v>4402.641</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="8" t="n">
         <v>-18572.367</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="8" t="n">
         <v>-26426.605</v>
       </c>
-      <c r="F6" s="21" t="n">
+      <c r="F6" s="20" t="n">
         <v>643.224</v>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="20" t="n">
         <v>14556.008</v>
       </c>
-      <c r="H6" s="21" t="n">
+      <c r="H6" s="20" t="n">
         <v>52394.883</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="20" t="n">
         <v>74368.942</v>
       </c>
-      <c r="J6" s="21" t="n">
+      <c r="J6" s="20" t="n">
         <v>155390.627</v>
       </c>
-      <c r="K6" s="20" t="n">
+      <c r="K6" s="8" t="n">
         <v>-12124.211</v>
       </c>
-      <c r="L6" s="21" t="n">
+      <c r="L6" s="20" t="n">
         <v>62936.723</v>
       </c>
-      <c r="M6" s="21" t="n">
+      <c r="M6" s="20" t="n">
         <v>75552.632</v>
       </c>
-      <c r="N6" s="21" t="n">
+      <c r="N6" s="20" t="n">
         <v>85156.228</v>
       </c>
-      <c r="O6" s="21" t="n">
+      <c r="O6" s="20" t="n">
         <v>25896.973</v>
       </c>
-      <c r="P6" s="20" t="n">
+      <c r="P6" s="8" t="n">
         <v>-22428.624</v>
       </c>
-      <c r="Q6" s="21" t="n">
+      <c r="Q6" s="20" t="n">
         <v>16274.839</v>
       </c>
-      <c r="R6" s="20" t="n">
+      <c r="R6" s="8" t="n">
         <v>-15037.71</v>
       </c>
-      <c r="S6" s="21" t="n">
+      <c r="S6" s="20" t="n">
         <v>32532.733</v>
       </c>
-      <c r="T6" s="21" t="n">
+      <c r="T6" s="20" t="n">
         <v>1396.743</v>
       </c>
-      <c r="U6" s="20" t="n">
+      <c r="U6" s="8" t="n">
         <v>-17348.77</v>
       </c>
-      <c r="V6" s="20" t="n">
+      <c r="V6" s="8" t="n">
         <v>-141168.328</v>
       </c>
-      <c r="W6" s="20" t="n">
+      <c r="W6" s="8" t="n">
         <v>-117733.553</v>
       </c>
-      <c r="X6" s="20" t="n">
+      <c r="X6" s="8" t="n">
         <v>-36630.77</v>
       </c>
-      <c r="Y6" s="20" t="n">
+      <c r="Y6" s="8" t="n">
         <v>-56620.783</v>
       </c>
-      <c r="Z6" s="21" t="n">
+      <c r="Z6" s="20" t="n">
         <v>78236.91</v>
       </c>
-      <c r="AA6" s="20" t="n">
+      <c r="AA6" s="8" t="n">
         <v>-212477.334</v>
       </c>
-      <c r="AB6" s="21" t="n">
+      <c r="AB6" s="20" t="n">
         <v>8357.906000000001</v>
       </c>
-      <c r="AC6" s="21" t="n">
+      <c r="AC6" s="20" t="n">
         <v>64261.805</v>
       </c>
     </row>
@@ -3053,271 +3059,271 @@
           <t>1809</t>
         </is>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="20" t="n">
         <v>21398.839</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="20" t="n">
         <v>41318.272</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="20" t="n">
         <v>90722.091</v>
       </c>
-      <c r="F7" s="21" t="n">
+      <c r="F7" s="20" t="n">
         <v>11180.802</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="20" t="n">
         <v>57838.483</v>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="20" t="n">
         <v>2808.482</v>
       </c>
-      <c r="I7" s="20" t="n">
+      <c r="I7" s="8" t="n">
         <v>-686.574</v>
       </c>
-      <c r="J7" s="20" t="n">
+      <c r="J7" s="8" t="n">
         <v>-73974.527</v>
       </c>
-      <c r="K7" s="21" t="n">
+      <c r="K7" s="20" t="n">
         <v>34058.554</v>
       </c>
-      <c r="L7" s="21" t="n">
+      <c r="L7" s="20" t="n">
         <v>11280.602</v>
       </c>
-      <c r="M7" s="21" t="n">
+      <c r="M7" s="20" t="n">
         <v>249513.458</v>
       </c>
-      <c r="N7" s="21" t="n">
+      <c r="N7" s="20" t="n">
         <v>70196.20299999999</v>
       </c>
-      <c r="O7" s="21" t="n">
+      <c r="O7" s="20" t="n">
         <v>5653.172</v>
       </c>
-      <c r="P7" s="21" t="n">
+      <c r="P7" s="20" t="n">
         <v>197242.065</v>
       </c>
-      <c r="Q7" s="20" t="n">
+      <c r="Q7" s="8" t="n">
         <v>-76307.204</v>
       </c>
-      <c r="R7" s="20" t="n">
+      <c r="R7" s="8" t="n">
         <v>-124016.063</v>
       </c>
-      <c r="S7" s="21" t="n">
+      <c r="S7" s="20" t="n">
         <v>32267.88</v>
       </c>
-      <c r="T7" s="20" t="n">
+      <c r="T7" s="8" t="n">
         <v>-26792.966</v>
       </c>
-      <c r="U7" s="21" t="n">
+      <c r="U7" s="20" t="n">
         <v>35093.592</v>
       </c>
-      <c r="V7" s="21" t="n">
+      <c r="V7" s="20" t="n">
         <v>227324.959</v>
       </c>
-      <c r="W7" s="20" t="n">
+      <c r="W7" s="8" t="n">
         <v>-630037.433</v>
       </c>
-      <c r="X7" s="21" t="n">
+      <c r="X7" s="20" t="n">
         <v>182431.271</v>
       </c>
-      <c r="Y7" s="21" t="n">
+      <c r="Y7" s="20" t="n">
         <v>437174.227</v>
       </c>
-      <c r="Z7" s="20" t="n">
+      <c r="Z7" s="8" t="n">
         <v>-56588.088</v>
       </c>
-      <c r="AA7" s="21" t="n">
+      <c r="AA7" s="20" t="n">
         <v>158704.826</v>
       </c>
-      <c r="AB7" s="21" t="n">
+      <c r="AB7" s="20" t="n">
         <v>54036.513</v>
       </c>
-      <c r="AC7" s="20" t="n">
+      <c r="AC7" s="8" t="n">
         <v>-72270.342</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">    Títulos — mercado primário</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="22" t="inlineStr">
         <is>
           <t>29004</t>
         </is>
       </c>
-      <c r="C8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="25" t="n">
+      <c r="C8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="8" t="n">
         <v>-123479.463</v>
       </c>
-      <c r="S8" s="26" t="n">
+      <c r="S8" s="24" t="n">
         <v>31896.944</v>
       </c>
-      <c r="T8" s="25" t="n">
+      <c r="T8" s="8" t="n">
         <v>-111168.532</v>
       </c>
-      <c r="U8" s="26" t="n">
+      <c r="U8" s="24" t="n">
         <v>32704.358</v>
       </c>
-      <c r="V8" s="25" t="n">
+      <c r="V8" s="8" t="n">
         <v>-15720.656</v>
       </c>
-      <c r="W8" s="25" t="n">
+      <c r="W8" s="8" t="n">
         <v>-365463.108</v>
       </c>
-      <c r="X8" s="25" t="n">
+      <c r="X8" s="8" t="n">
         <v>-121550.764</v>
       </c>
-      <c r="Y8" s="26" t="n">
+      <c r="Y8" s="24" t="n">
         <v>251182.278</v>
       </c>
-      <c r="Z8" s="26" t="n">
+      <c r="Z8" s="24" t="n">
         <v>73732.46000000001</v>
       </c>
-      <c r="AA8" s="26" t="n">
+      <c r="AA8" s="24" t="n">
         <v>65135.039</v>
       </c>
-      <c r="AB8" s="25" t="n">
+      <c r="AB8" s="8" t="n">
         <v>-376560.608</v>
       </c>
-      <c r="AC8" s="26" t="n">
+      <c r="AC8" s="24" t="n">
         <v>127370.052</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">    Títulos — mercado secundário</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>29006</t>
         </is>
       </c>
-      <c r="C9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" s="25" t="n">
+      <c r="C9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="8" t="n">
         <v>-536.6</v>
       </c>
-      <c r="S9" s="26" t="n">
+      <c r="S9" s="24" t="n">
         <v>370.936</v>
       </c>
-      <c r="T9" s="26" t="n">
+      <c r="T9" s="24" t="n">
         <v>84375.56600000001</v>
       </c>
-      <c r="U9" s="26" t="n">
+      <c r="U9" s="24" t="n">
         <v>2389.234</v>
       </c>
-      <c r="V9" s="26" t="n">
+      <c r="V9" s="24" t="n">
         <v>243045.615</v>
       </c>
-      <c r="W9" s="25" t="n">
+      <c r="W9" s="8" t="n">
         <v>-264574.325</v>
       </c>
-      <c r="X9" s="26" t="n">
+      <c r="X9" s="24" t="n">
         <v>303982.035</v>
       </c>
-      <c r="Y9" s="26" t="n">
+      <c r="Y9" s="24" t="n">
         <v>185991.949</v>
       </c>
-      <c r="Z9" s="25" t="n">
+      <c r="Z9" s="8" t="n">
         <v>-130320.548</v>
       </c>
-      <c r="AA9" s="26" t="n">
+      <c r="AA9" s="24" t="n">
         <v>93569.787</v>
       </c>
-      <c r="AB9" s="26" t="n">
+      <c r="AB9" s="24" t="n">
         <v>430597.121</v>
       </c>
-      <c r="AC9" s="25" t="n">
+      <c r="AC9" s="8" t="n">
         <v>-199640.393</v>
       </c>
     </row>
@@ -3332,85 +3338,85 @@
           <t>1815</t>
         </is>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="20" t="n">
         <v>1478.559</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="8" t="n">
         <v>-1806.911</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="8" t="n">
         <v>-33769.655</v>
       </c>
-      <c r="F10" s="21" t="n">
+      <c r="F10" s="20" t="n">
         <v>6729.147</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="8" t="n">
         <v>-2400.391</v>
       </c>
-      <c r="H10" s="21" t="n">
+      <c r="H10" s="20" t="n">
         <v>2373.784</v>
       </c>
-      <c r="I10" s="20" t="n">
+      <c r="I10" s="8" t="n">
         <v>-764.37</v>
       </c>
-      <c r="J10" s="20" t="n">
+      <c r="J10" s="8" t="n">
         <v>-10600.939</v>
       </c>
-      <c r="K10" s="21" t="n">
+      <c r="K10" s="20" t="n">
         <v>57041.22</v>
       </c>
-      <c r="L10" s="20" t="n">
+      <c r="L10" s="8" t="n">
         <v>-3425.469</v>
       </c>
-      <c r="M10" s="20" t="n">
+      <c r="M10" s="8" t="n">
         <v>-236911.071</v>
       </c>
-      <c r="N10" s="20" t="n">
+      <c r="N10" s="8" t="n">
         <v>-24388.014</v>
       </c>
-      <c r="O10" s="21" t="n">
+      <c r="O10" s="20" t="n">
         <v>118682.701</v>
       </c>
-      <c r="P10" s="20" t="n">
+      <c r="P10" s="8" t="n">
         <v>-19903.346</v>
       </c>
-      <c r="Q10" s="21" t="n">
+      <c r="Q10" s="20" t="n">
         <v>56163.369</v>
       </c>
-      <c r="R10" s="20" t="n">
+      <c r="R10" s="8" t="n">
         <v>-24740.332</v>
       </c>
-      <c r="S10" s="21" t="n">
+      <c r="S10" s="20" t="n">
         <v>6054.528</v>
       </c>
-      <c r="T10" s="21" t="n">
+      <c r="T10" s="20" t="n">
         <v>867.627</v>
       </c>
-      <c r="U10" s="21" t="n">
+      <c r="U10" s="20" t="n">
         <v>13987.567</v>
       </c>
-      <c r="V10" s="21" t="n">
+      <c r="V10" s="20" t="n">
         <v>16690.766</v>
       </c>
-      <c r="W10" s="21" t="n">
+      <c r="W10" s="20" t="n">
         <v>69829.095</v>
       </c>
-      <c r="X10" s="20" t="n">
+      <c r="X10" s="8" t="n">
         <v>-26059.891</v>
       </c>
-      <c r="Y10" s="20" t="n">
+      <c r="Y10" s="8" t="n">
         <v>-54168.5</v>
       </c>
-      <c r="Z10" s="20" t="n">
+      <c r="Z10" s="8" t="n">
         <v>-45370.899</v>
       </c>
-      <c r="AA10" s="20" t="n">
+      <c r="AA10" s="8" t="n">
         <v>-706.95</v>
       </c>
-      <c r="AB10" s="21" t="n">
+      <c r="AB10" s="20" t="n">
         <v>45376.981</v>
       </c>
-      <c r="AC10" s="21" t="n">
+      <c r="AC10" s="20" t="n">
         <v>26591.66</v>
       </c>
     </row>
@@ -3425,85 +3431,85 @@
           <t>12484</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="8" t="n">
         <v>-614.971</v>
       </c>
-      <c r="D11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="21" t="n">
+      <c r="D11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="20" t="n">
         <v>400.375</v>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" s="20" t="n">
         <v>2.247</v>
       </c>
-      <c r="G11" s="20" t="n">
+      <c r="G11" s="8" t="n">
         <v>-7.14</v>
       </c>
-      <c r="H11" s="20" t="n">
+      <c r="H11" s="8" t="n">
         <v>-3.343</v>
       </c>
-      <c r="I11" s="20" t="n">
+      <c r="I11" s="8" t="n">
         <v>-1.476</v>
       </c>
-      <c r="J11" s="20" t="n">
+      <c r="J11" s="8" t="n">
         <v>-3.017</v>
       </c>
-      <c r="K11" s="20" t="n">
+      <c r="K11" s="8" t="n">
         <v>-1.073</v>
       </c>
-      <c r="L11" s="20" t="n">
+      <c r="L11" s="8" t="n">
         <v>-1.181</v>
       </c>
-      <c r="M11" s="20" t="n">
+      <c r="M11" s="8" t="n">
         <v>-0.539</v>
       </c>
-      <c r="N11" s="20" t="n">
+      <c r="N11" s="8" t="n">
         <v>-0.5600000000000001</v>
       </c>
-      <c r="O11" s="21" t="n">
+      <c r="O11" s="20" t="n">
         <v>45.943</v>
       </c>
-      <c r="P11" s="20" t="n">
+      <c r="P11" s="8" t="n">
         <v>-1.675</v>
       </c>
-      <c r="Q11" s="20" t="n">
+      <c r="Q11" s="8" t="n">
         <v>-0.045</v>
       </c>
-      <c r="R11" s="20" t="n">
+      <c r="R11" s="8" t="n">
         <v>-0.593</v>
       </c>
-      <c r="S11" s="20" t="n">
+      <c r="S11" s="8" t="n">
         <v>-3.179</v>
       </c>
-      <c r="T11" s="20" t="n">
+      <c r="T11" s="8" t="n">
         <v>-0.181</v>
       </c>
-      <c r="U11" s="21" t="n">
+      <c r="U11" s="20" t="n">
         <v>13.2</v>
       </c>
-      <c r="V11" s="20" t="n">
+      <c r="V11" s="8" t="n">
         <v>-14.549</v>
       </c>
-      <c r="W11" s="21" t="n">
+      <c r="W11" s="20" t="n">
         <v>3.485</v>
       </c>
-      <c r="X11" s="21" t="n">
+      <c r="X11" s="20" t="n">
         <v>44.99</v>
       </c>
-      <c r="Y11" s="20" t="n">
+      <c r="Y11" s="8" t="n">
         <v>-27.398</v>
       </c>
-      <c r="Z11" s="20" t="n">
+      <c r="Z11" s="8" t="n">
         <v>-29.715</v>
       </c>
-      <c r="AA11" s="20" t="n">
+      <c r="AA11" s="8" t="n">
         <v>-0.788</v>
       </c>
-      <c r="AB11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC11" s="27" t="n">
+      <c r="AB11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3518,85 +3524,85 @@
           <t>12487</t>
         </is>
       </c>
-      <c r="C12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="21" t="n">
+      <c r="C12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="20" t="n">
         <v>10942.004</v>
       </c>
-      <c r="F12" s="20" t="n">
+      <c r="F12" s="8" t="n">
         <v>-15632.065</v>
       </c>
-      <c r="G12" s="20" t="n">
+      <c r="G12" s="8" t="n">
         <v>-6032.014</v>
       </c>
-      <c r="H12" s="20" t="n">
+      <c r="H12" s="8" t="n">
         <v>-2684.423</v>
       </c>
-      <c r="I12" s="21" t="n">
+      <c r="I12" s="20" t="n">
         <v>5436.454</v>
       </c>
-      <c r="J12" s="21" t="n">
+      <c r="J12" s="20" t="n">
         <v>8812.156000000001</v>
       </c>
-      <c r="K12" s="20" t="n">
+      <c r="K12" s="8" t="n">
         <v>-4801.25</v>
       </c>
-      <c r="L12" s="20" t="n">
+      <c r="L12" s="8" t="n">
         <v>-3198.916</v>
       </c>
-      <c r="M12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="20" t="n">
+      <c r="M12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>-705.683</v>
       </c>
-      <c r="O12" s="20" t="n">
+      <c r="O12" s="8" t="n">
         <v>-1100.801</v>
       </c>
-      <c r="P12" s="21" t="n">
+      <c r="P12" s="20" t="n">
         <v>1314.564</v>
       </c>
-      <c r="Q12" s="21" t="n">
+      <c r="Q12" s="20" t="n">
         <v>17329.053</v>
       </c>
-      <c r="R12" s="21" t="n">
+      <c r="R12" s="20" t="n">
         <v>89657.15300000001</v>
       </c>
-      <c r="S12" s="20" t="n">
+      <c r="S12" s="8" t="n">
         <v>-75562.37300000001</v>
       </c>
-      <c r="T12" s="20" t="n">
+      <c r="T12" s="8" t="n">
         <v>-7032.535</v>
       </c>
-      <c r="U12" s="21" t="n">
+      <c r="U12" s="20" t="n">
         <v>15125.016</v>
       </c>
-      <c r="V12" s="21" t="n">
+      <c r="V12" s="20" t="n">
         <v>7639.551</v>
       </c>
-      <c r="W12" s="21" t="n">
+      <c r="W12" s="20" t="n">
         <v>40800.821</v>
       </c>
-      <c r="X12" s="21" t="n">
+      <c r="X12" s="20" t="n">
         <v>22323.949</v>
       </c>
-      <c r="Y12" s="20" t="n">
+      <c r="Y12" s="8" t="n">
         <v>-92265.39999999999</v>
       </c>
-      <c r="Z12" s="20" t="n">
+      <c r="Z12" s="8" t="n">
         <v>-70871.662</v>
       </c>
-      <c r="AA12" s="21" t="n">
+      <c r="AA12" s="20" t="n">
         <v>115930.245</v>
       </c>
-      <c r="AB12" s="20" t="n">
+      <c r="AB12" s="8" t="n">
         <v>-105895.906</v>
       </c>
-      <c r="AC12" s="20" t="n">
+      <c r="AC12" s="8" t="n">
         <v>-74564.97500000001</v>
       </c>
     </row>
@@ -3611,85 +3617,85 @@
           <t>28724</t>
         </is>
       </c>
-      <c r="C13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="W13" s="21" t="n">
+      <c r="C13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" s="20" t="n">
         <v>67236.04399999999</v>
       </c>
-      <c r="X13" s="20" t="n">
+      <c r="X13" s="8" t="n">
         <v>-52769.578</v>
       </c>
-      <c r="Y13" s="21" t="n">
+      <c r="Y13" s="20" t="n">
         <v>9097.299000000001</v>
       </c>
-      <c r="Z13" s="20" t="n">
+      <c r="Z13" s="8" t="n">
         <v>-33737.198</v>
       </c>
-      <c r="AA13" s="20" t="n">
+      <c r="AA13" s="8" t="n">
         <v>-0.021</v>
       </c>
-      <c r="AB13" s="20" t="n">
+      <c r="AB13" s="8" t="n">
         <v>-0.024</v>
       </c>
-      <c r="AC13" s="20" t="n">
+      <c r="AC13" s="8" t="n">
         <v>-5.306</v>
       </c>
     </row>
@@ -3704,193 +3710,193 @@
           <t>1818</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="8" t="n">
         <v>-839.2619999999999</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="8" t="n">
         <v>-3424.281</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="8" t="n">
         <v>-1338.211</v>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="8" t="n">
         <v>-1941.998</v>
       </c>
-      <c r="G14" s="20" t="n">
+      <c r="G14" s="8" t="n">
         <v>-148.935</v>
       </c>
-      <c r="H14" s="21" t="n">
+      <c r="H14" s="20" t="n">
         <v>632.9059999999999</v>
       </c>
-      <c r="I14" s="21" t="n">
+      <c r="I14" s="20" t="n">
         <v>1012.499</v>
       </c>
-      <c r="J14" s="21" t="n">
+      <c r="J14" s="20" t="n">
         <v>1491.448</v>
       </c>
-      <c r="K14" s="21" t="n">
+      <c r="K14" s="20" t="n">
         <v>1071.994</v>
       </c>
-      <c r="L14" s="21" t="n">
+      <c r="L14" s="20" t="n">
         <v>3242.878</v>
       </c>
-      <c r="M14" s="21" t="n">
+      <c r="M14" s="20" t="n">
         <v>3829.68</v>
       </c>
-      <c r="N14" s="21" t="n">
+      <c r="N14" s="20" t="n">
         <v>2756.678</v>
       </c>
-      <c r="O14" s="20" t="n">
+      <c r="O14" s="8" t="n">
         <v>-8392.875</v>
       </c>
-      <c r="P14" s="20" t="n">
+      <c r="P14" s="8" t="n">
         <v>-12532.941</v>
       </c>
-      <c r="Q14" s="21" t="n">
+      <c r="Q14" s="20" t="n">
         <v>1227.406</v>
       </c>
-      <c r="R14" s="21" t="n">
+      <c r="R14" s="20" t="n">
         <v>6233.098</v>
       </c>
-      <c r="S14" s="21" t="n">
+      <c r="S14" s="20" t="n">
         <v>7424.617</v>
       </c>
-      <c r="T14" s="21" t="n">
+      <c r="T14" s="20" t="n">
         <v>5896.818</v>
       </c>
-      <c r="U14" s="21" t="n">
+      <c r="U14" s="20" t="n">
         <v>2909.758</v>
       </c>
-      <c r="V14" s="20" t="n">
+      <c r="V14" s="8" t="n">
         <v>-6634.019</v>
       </c>
-      <c r="W14" s="20" t="n">
+      <c r="W14" s="8" t="n">
         <v>-19343.055</v>
       </c>
-      <c r="X14" s="20" t="n">
+      <c r="X14" s="8" t="n">
         <v>-30402.627</v>
       </c>
-      <c r="Y14" s="20" t="n">
+      <c r="Y14" s="8" t="n">
         <v>-80194.454</v>
       </c>
-      <c r="Z14" s="20" t="n">
+      <c r="Z14" s="8" t="n">
         <v>-75435.61500000001</v>
       </c>
-      <c r="AA14" s="20" t="n">
+      <c r="AA14" s="8" t="n">
         <v>-98786.795</v>
       </c>
-      <c r="AB14" s="20" t="n">
+      <c r="AB14" s="8" t="n">
         <v>-100762.164</v>
       </c>
-      <c r="AC14" s="20" t="n">
+      <c r="AC14" s="8" t="n">
         <v>-133484.659</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Variação da base (= soma dos fatores)</t>
         </is>
       </c>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>Σ</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="28" t="n">
         <v>-713.342</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="13" t="n">
         <v>5569.787</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="13" t="n">
         <v>20046.302</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F15" s="28" t="n">
         <v>-83.136</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="13" t="n">
         <v>15513.541</v>
       </c>
-      <c r="H15" s="11" t="n">
+      <c r="H15" s="13" t="n">
         <v>12514.558</v>
       </c>
-      <c r="I15" s="11" t="n">
+      <c r="I15" s="13" t="n">
         <v>19854.766</v>
       </c>
-      <c r="J15" s="11" t="n">
+      <c r="J15" s="13" t="n">
         <v>25514.866</v>
       </c>
-      <c r="K15" s="11" t="n">
+      <c r="K15" s="13" t="n">
         <v>932.838</v>
       </c>
-      <c r="L15" s="11" t="n">
+      <c r="L15" s="13" t="n">
         <v>18523.13</v>
       </c>
-      <c r="M15" s="11" t="n">
+      <c r="M15" s="13" t="n">
         <v>40780.487</v>
       </c>
-      <c r="N15" s="11" t="n">
+      <c r="N15" s="13" t="n">
         <v>7381.989</v>
       </c>
-      <c r="O15" s="11" t="n">
+      <c r="O15" s="13" t="n">
         <v>19136.141</v>
       </c>
-      <c r="P15" s="11" t="n">
+      <c r="P15" s="13" t="n">
         <v>16135.254</v>
       </c>
-      <c r="Q15" s="11" t="n">
+      <c r="Q15" s="13" t="n">
         <v>14018.932</v>
       </c>
-      <c r="R15" s="11" t="n">
+      <c r="R15" s="28" t="n">
         <v>-8238.638999999999</v>
       </c>
-      <c r="S15" s="11" t="n">
+      <c r="S15" s="13" t="n">
         <v>14998.397</v>
       </c>
-      <c r="T15" s="11" t="n">
+      <c r="T15" s="13" t="n">
         <v>26468.383</v>
       </c>
-      <c r="U15" s="11" t="n">
+      <c r="U15" s="13" t="n">
         <v>5294.233</v>
       </c>
-      <c r="V15" s="11" t="n">
+      <c r="V15" s="13" t="n">
         <v>14537.328</v>
       </c>
-      <c r="W15" s="11" t="n">
+      <c r="W15" s="13" t="n">
         <v>114949.942</v>
       </c>
-      <c r="X15" s="11" t="n">
+      <c r="X15" s="28" t="n">
         <v>-22353.137</v>
       </c>
-      <c r="Y15" s="11" t="n">
+      <c r="Y15" s="13" t="n">
         <v>10476.4</v>
       </c>
-      <c r="Z15" s="11" t="n">
+      <c r="Z15" s="13" t="n">
         <v>3058.705</v>
       </c>
-      <c r="AA15" s="11" t="n">
+      <c r="AA15" s="13" t="n">
         <v>28495.118</v>
       </c>
-      <c r="AB15" s="11" t="n">
+      <c r="AB15" s="28" t="n">
         <v>-4116.189</v>
       </c>
-      <c r="AC15" s="11" t="n">
+      <c r="AC15" s="28" t="n">
         <v>-14645.627</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>Memória: Δ estoque da base (fim a fim)</t>
         </is>
       </c>
-      <c r="B16" s="31" t="inlineStr">
+      <c r="B16" s="30" t="inlineStr">
         <is>
           <t>Δ</t>
         </is>
       </c>
-      <c r="C16" s="32" t="n">
+      <c r="C16" s="31" t="n">
         <v>-743.944</v>
       </c>
       <c r="D16" s="32" t="n">
@@ -3899,7 +3905,7 @@
       <c r="E16" s="32" t="n">
         <v>20046.301</v>
       </c>
-      <c r="F16" s="32" t="n">
+      <c r="F16" s="31" t="n">
         <v>-83.136</v>
       </c>
       <c r="G16" s="32" t="n">
@@ -3935,7 +3941,7 @@
       <c r="Q16" s="32" t="n">
         <v>14018.739</v>
       </c>
-      <c r="R16" s="32" t="n">
+      <c r="R16" s="31" t="n">
         <v>-8239.594999999999</v>
       </c>
       <c r="S16" s="32" t="n">
@@ -3953,7 +3959,7 @@
       <c r="W16" s="32" t="n">
         <v>114949.946</v>
       </c>
-      <c r="X16" s="32" t="n">
+      <c r="X16" s="31" t="n">
         <v>-22353.134</v>
       </c>
       <c r="Y16" s="32" t="n">
@@ -3965,20 +3971,20 @@
       <c r="AA16" s="32" t="n">
         <v>28494.96</v>
       </c>
-      <c r="AB16" s="32" t="n">
+      <c r="AB16" s="31" t="n">
         <v>-4116.934</v>
       </c>
-      <c r="AC16" s="32" t="n">
+      <c r="AC16" s="31" t="n">
         <v>-14544.967</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>Memória: resíduo (soma − Δ estoque)</t>
         </is>
       </c>
-      <c r="B17" s="31" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>ε</t>
         </is>
@@ -4022,7 +4028,7 @@
       <c r="O17" s="32" t="n">
         <v>0</v>
       </c>
-      <c r="P17" s="32" t="n">
+      <c r="P17" s="31" t="n">
         <v>-3.072</v>
       </c>
       <c r="Q17" s="32" t="n">
@@ -4043,16 +4049,16 @@
       <c r="V17" s="32" t="n">
         <v>0.082</v>
       </c>
-      <c r="W17" s="32" t="n">
+      <c r="W17" s="31" t="n">
         <v>-0.004</v>
       </c>
-      <c r="X17" s="32" t="n">
+      <c r="X17" s="31" t="n">
         <v>-0.003</v>
       </c>
       <c r="Y17" s="32" t="n">
         <v>0.001</v>
       </c>
-      <c r="Z17" s="32" t="n">
+      <c r="Z17" s="31" t="n">
         <v>-0.005</v>
       </c>
       <c r="AA17" s="32" t="n">
@@ -4061,7 +4067,7 @@
       <c r="AB17" s="32" t="n">
         <v>0.745</v>
       </c>
-      <c r="AC17" s="32" t="n">
+      <c r="AC17" s="31" t="n">
         <v>-100.66</v>
       </c>
     </row>
@@ -4076,85 +4082,85 @@
           <t>1788</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="11" t="n">
         <v>47686.213</v>
       </c>
-      <c r="D18" s="12" t="n">
+      <c r="D18" s="11" t="n">
         <v>53255.971</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="11" t="n">
         <v>73302.272</v>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F18" s="11" t="n">
         <v>73219.136</v>
       </c>
-      <c r="G18" s="12" t="n">
+      <c r="G18" s="11" t="n">
         <v>88732.677</v>
       </c>
-      <c r="H18" s="12" t="n">
+      <c r="H18" s="11" t="n">
         <v>101247.235</v>
       </c>
-      <c r="I18" s="12" t="n">
+      <c r="I18" s="11" t="n">
         <v>121102.001</v>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="11" t="n">
         <v>146616.867</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="K18" s="11" t="n">
         <v>147549.705</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="L18" s="11" t="n">
         <v>166072.835</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="M18" s="11" t="n">
         <v>206853.322</v>
       </c>
-      <c r="N18" s="12" t="n">
+      <c r="N18" s="11" t="n">
         <v>214235.311</v>
       </c>
-      <c r="O18" s="12" t="n">
+      <c r="O18" s="11" t="n">
         <v>233371.452</v>
       </c>
-      <c r="P18" s="12" t="n">
+      <c r="P18" s="11" t="n">
         <v>249509.778</v>
       </c>
-      <c r="Q18" s="12" t="n">
+      <c r="Q18" s="11" t="n">
         <v>263528.517</v>
       </c>
-      <c r="R18" s="12" t="n">
+      <c r="R18" s="11" t="n">
         <v>255288.922</v>
       </c>
-      <c r="S18" s="12" t="n">
+      <c r="S18" s="11" t="n">
         <v>270287.146</v>
       </c>
-      <c r="T18" s="12" t="n">
+      <c r="T18" s="11" t="n">
         <v>296755.456</v>
       </c>
-      <c r="U18" s="12" t="n">
+      <c r="U18" s="11" t="n">
         <v>302049.461</v>
       </c>
-      <c r="V18" s="12" t="n">
+      <c r="V18" s="11" t="n">
         <v>316586.707</v>
       </c>
-      <c r="W18" s="12" t="n">
+      <c r="W18" s="11" t="n">
         <v>431536.653</v>
       </c>
-      <c r="X18" s="12" t="n">
+      <c r="X18" s="11" t="n">
         <v>409183.519</v>
       </c>
-      <c r="Y18" s="12" t="n">
+      <c r="Y18" s="11" t="n">
         <v>419659.918</v>
       </c>
-      <c r="Z18" s="12" t="n">
+      <c r="Z18" s="11" t="n">
         <v>422718.628</v>
       </c>
-      <c r="AA18" s="12" t="n">
+      <c r="AA18" s="11" t="n">
         <v>451213.588</v>
       </c>
-      <c r="AB18" s="12" t="n">
+      <c r="AB18" s="11" t="n">
         <v>447096.654</v>
       </c>
-      <c r="AC18" s="12" t="n">
+      <c r="AC18" s="11" t="n">
         <v>432551.687</v>
       </c>
     </row>
@@ -4169,85 +4175,85 @@
           <t>1786</t>
         </is>
       </c>
-      <c r="C19" s="27" t="n">
+      <c r="C19" s="25" t="n">
         <v>32633.056</v>
       </c>
-      <c r="D19" s="27" t="n">
+      <c r="D19" s="25" t="n">
         <v>37668.836</v>
       </c>
-      <c r="E19" s="27" t="n">
+      <c r="E19" s="25" t="n">
         <v>49931.066</v>
       </c>
-      <c r="F19" s="27" t="n">
+      <c r="F19" s="25" t="n">
         <v>51363.863</v>
       </c>
-      <c r="G19" s="27" t="n">
+      <c r="G19" s="25" t="n">
         <v>61935.635</v>
       </c>
-      <c r="H19" s="27" t="n">
+      <c r="H19" s="25" t="n">
         <v>70033.641</v>
       </c>
-      <c r="I19" s="27" t="n">
+      <c r="I19" s="25" t="n">
         <v>85824.753</v>
       </c>
-      <c r="J19" s="27" t="n">
+      <c r="J19" s="25" t="n">
         <v>102885.047</v>
       </c>
-      <c r="K19" s="27" t="n">
+      <c r="K19" s="25" t="n">
         <v>115590.704</v>
       </c>
-      <c r="L19" s="27" t="n">
+      <c r="L19" s="25" t="n">
         <v>131861.185</v>
       </c>
-      <c r="M19" s="27" t="n">
+      <c r="M19" s="25" t="n">
         <v>151145.368</v>
       </c>
-      <c r="N19" s="27" t="n">
+      <c r="N19" s="25" t="n">
         <v>162769.67</v>
       </c>
-      <c r="O19" s="27" t="n">
+      <c r="O19" s="25" t="n">
         <v>187434.736</v>
       </c>
-      <c r="P19" s="27" t="n">
+      <c r="P19" s="25" t="n">
         <v>204052.42</v>
       </c>
-      <c r="Q19" s="27" t="n">
+      <c r="Q19" s="25" t="n">
         <v>220853.706</v>
       </c>
-      <c r="R19" s="27" t="n">
+      <c r="R19" s="25" t="n">
         <v>225485.184</v>
       </c>
-      <c r="S19" s="27" t="n">
+      <c r="S19" s="25" t="n">
         <v>232145.593</v>
       </c>
-      <c r="T19" s="27" t="n">
+      <c r="T19" s="25" t="n">
         <v>250363.681</v>
       </c>
-      <c r="U19" s="27" t="n">
+      <c r="U19" s="25" t="n">
         <v>264967.669</v>
       </c>
-      <c r="V19" s="27" t="n">
+      <c r="V19" s="25" t="n">
         <v>280685.185</v>
       </c>
-      <c r="W19" s="27" t="n">
+      <c r="W19" s="25" t="n">
         <v>370441.036</v>
       </c>
-      <c r="X19" s="27" t="n">
+      <c r="X19" s="25" t="n">
         <v>339013.043</v>
       </c>
-      <c r="Y19" s="27" t="n">
+      <c r="Y19" s="25" t="n">
         <v>342334.138</v>
       </c>
-      <c r="Z19" s="27" t="n">
+      <c r="Z19" s="25" t="n">
         <v>341616.828</v>
       </c>
-      <c r="AA19" s="27" t="n">
+      <c r="AA19" s="25" t="n">
         <v>355858.101</v>
       </c>
-      <c r="AB19" s="27" t="n">
+      <c r="AB19" s="25" t="n">
         <v>368625.466</v>
       </c>
-      <c r="AC19" s="27" t="n">
+      <c r="AC19" s="25" t="n">
         <v>382994.849</v>
       </c>
     </row>
@@ -4262,85 +4268,85 @@
           <t>1787</t>
         </is>
       </c>
-      <c r="C20" s="27" t="n">
+      <c r="C20" s="25" t="n">
         <v>15053.157</v>
       </c>
-      <c r="D20" s="27" t="n">
+      <c r="D20" s="25" t="n">
         <v>15587.135</v>
       </c>
-      <c r="E20" s="27" t="n">
+      <c r="E20" s="25" t="n">
         <v>23371.206</v>
       </c>
-      <c r="F20" s="27" t="n">
+      <c r="F20" s="25" t="n">
         <v>21855.273</v>
       </c>
-      <c r="G20" s="27" t="n">
+      <c r="G20" s="25" t="n">
         <v>26797.042</v>
       </c>
-      <c r="H20" s="27" t="n">
+      <c r="H20" s="25" t="n">
         <v>31213.594</v>
       </c>
-      <c r="I20" s="27" t="n">
+      <c r="I20" s="25" t="n">
         <v>35277.248</v>
       </c>
-      <c r="J20" s="27" t="n">
+      <c r="J20" s="25" t="n">
         <v>43731.82</v>
       </c>
-      <c r="K20" s="27" t="n">
+      <c r="K20" s="25" t="n">
         <v>31959.001</v>
       </c>
-      <c r="L20" s="27" t="n">
+      <c r="L20" s="25" t="n">
         <v>34211.65</v>
       </c>
-      <c r="M20" s="27" t="n">
+      <c r="M20" s="25" t="n">
         <v>55707.954</v>
       </c>
-      <c r="N20" s="27" t="n">
+      <c r="N20" s="25" t="n">
         <v>51465.641</v>
       </c>
-      <c r="O20" s="27" t="n">
+      <c r="O20" s="25" t="n">
         <v>45936.716</v>
       </c>
-      <c r="P20" s="27" t="n">
+      <c r="P20" s="25" t="n">
         <v>45457.358</v>
       </c>
-      <c r="Q20" s="27" t="n">
+      <c r="Q20" s="25" t="n">
         <v>42674.811</v>
       </c>
-      <c r="R20" s="27" t="n">
+      <c r="R20" s="25" t="n">
         <v>29803.738</v>
       </c>
-      <c r="S20" s="27" t="n">
+      <c r="S20" s="25" t="n">
         <v>38141.553</v>
       </c>
-      <c r="T20" s="27" t="n">
+      <c r="T20" s="25" t="n">
         <v>46391.775</v>
       </c>
-      <c r="U20" s="27" t="n">
+      <c r="U20" s="25" t="n">
         <v>37081.792</v>
       </c>
-      <c r="V20" s="27" t="n">
+      <c r="V20" s="25" t="n">
         <v>35901.522</v>
       </c>
-      <c r="W20" s="27" t="n">
+      <c r="W20" s="25" t="n">
         <v>61095.617</v>
       </c>
-      <c r="X20" s="27" t="n">
+      <c r="X20" s="25" t="n">
         <v>70170.476</v>
       </c>
-      <c r="Y20" s="27" t="n">
+      <c r="Y20" s="25" t="n">
         <v>77325.78</v>
       </c>
-      <c r="Z20" s="27" t="n">
+      <c r="Z20" s="25" t="n">
         <v>81101.8</v>
       </c>
-      <c r="AA20" s="27" t="n">
+      <c r="AA20" s="25" t="n">
         <v>95355.488</v>
       </c>
-      <c r="AB20" s="27" t="n">
+      <c r="AB20" s="25" t="n">
         <v>78471.18799999999</v>
       </c>
-      <c r="AC20" s="27" t="n">
+      <c r="AC20" s="25" t="n">
         <v>49556.839</v>
       </c>
     </row>
@@ -4572,85 +4578,85 @@
       <c r="B5" s="19" t="n">
         <v>1810</v>
       </c>
-      <c r="C5" s="20" t="n">
+      <c r="C5" s="8" t="n">
         <v>-90.184</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="20" t="n">
         <v>8397.878000000001</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="20" t="n">
         <v>196.734</v>
       </c>
-      <c r="F5" s="21" t="n">
+      <c r="F5" s="20" t="n">
         <v>11711.648</v>
       </c>
-      <c r="G5" s="20" t="n">
+      <c r="G5" s="8" t="n">
         <v>-2788.872</v>
       </c>
-      <c r="H5" s="20" t="n">
+      <c r="H5" s="8" t="n">
         <v>-1519.602</v>
       </c>
-      <c r="I5" s="20" t="n">
+      <c r="I5" s="8" t="n">
         <v>-2159.061</v>
       </c>
-      <c r="J5" s="20" t="n">
+      <c r="J5" s="8" t="n">
         <v>-4826.282</v>
       </c>
-      <c r="K5" s="20" t="n">
+      <c r="K5" s="8" t="n">
         <v>-3477.074</v>
       </c>
-      <c r="L5" s="20" t="n">
+      <c r="L5" s="8" t="n">
         <v>-15185.319</v>
       </c>
-      <c r="M5" s="20" t="n">
+      <c r="M5" s="8" t="n">
         <v>-22880.052</v>
       </c>
-      <c r="N5" s="20" t="n">
+      <c r="N5" s="8" t="n">
         <v>-17945.76</v>
       </c>
-      <c r="O5" s="20" t="n">
+      <c r="O5" s="8" t="n">
         <v>-39380.522</v>
       </c>
-      <c r="P5" s="20" t="n">
+      <c r="P5" s="8" t="n">
         <v>-43098.963</v>
       </c>
-      <c r="Q5" s="20" t="n">
+      <c r="Q5" s="8" t="n">
         <v>-17938.494</v>
       </c>
-      <c r="R5" s="21" t="n">
+      <c r="R5" s="20" t="n">
         <v>31966.901</v>
       </c>
-      <c r="S5" s="20" t="n">
+      <c r="S5" s="8" t="n">
         <v>-52397.634</v>
       </c>
-      <c r="T5" s="21" t="n">
+      <c r="T5" s="20" t="n">
         <v>7163.59</v>
       </c>
-      <c r="U5" s="21" t="n">
+      <c r="U5" s="20" t="n">
         <v>20453.395</v>
       </c>
-      <c r="V5" s="20" t="n">
+      <c r="V5" s="8" t="n">
         <v>-43975.649</v>
       </c>
-      <c r="W5" s="21" t="n">
+      <c r="W5" s="20" t="n">
         <v>25213.146</v>
       </c>
-      <c r="X5" s="20" t="n">
+      <c r="X5" s="8" t="n">
         <v>-42883.828</v>
       </c>
-      <c r="Y5" s="20" t="n">
+      <c r="Y5" s="8" t="n">
         <v>-35780.006</v>
       </c>
-      <c r="Z5" s="21" t="n">
+      <c r="Z5" s="20" t="n">
         <v>80331.787</v>
       </c>
-      <c r="AA5" s="20" t="n">
+      <c r="AA5" s="8" t="n">
         <v>-55712.578</v>
       </c>
-      <c r="AB5" s="20" t="n">
+      <c r="AB5" s="8" t="n">
         <v>-35402.732</v>
       </c>
-      <c r="AC5" s="21" t="n">
+      <c r="AC5" s="20" t="n">
         <v>43000.983</v>
       </c>
     </row>
@@ -4663,85 +4669,85 @@
       <c r="B6" s="19" t="n">
         <v>1811</v>
       </c>
-      <c r="C6" s="20" t="n">
+      <c r="C6" s="8" t="n">
         <v>-1941.905</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="8" t="n">
         <v>-2232.312</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="8" t="n">
         <v>-4981.6</v>
       </c>
-      <c r="F6" s="21" t="n">
+      <c r="F6" s="20" t="n">
         <v>13.499</v>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="20" t="n">
         <v>7186.047</v>
       </c>
-      <c r="H6" s="21" t="n">
+      <c r="H6" s="20" t="n">
         <v>9261.061</v>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="20" t="n">
         <v>5568.509</v>
       </c>
-      <c r="J6" s="21" t="n">
+      <c r="J6" s="20" t="n">
         <v>4210.354</v>
       </c>
-      <c r="K6" s="20" t="n">
+      <c r="K6" s="8" t="n">
         <v>-7846.766</v>
       </c>
-      <c r="L6" s="21" t="n">
+      <c r="L6" s="20" t="n">
         <v>6337.003</v>
       </c>
-      <c r="M6" s="21" t="n">
+      <c r="M6" s="20" t="n">
         <v>4276.126</v>
       </c>
-      <c r="N6" s="21" t="n">
+      <c r="N6" s="20" t="n">
         <v>303.625</v>
       </c>
-      <c r="O6" s="20" t="n">
+      <c r="O6" s="8" t="n">
         <v>-10975.444</v>
       </c>
-      <c r="P6" s="20" t="n">
+      <c r="P6" s="8" t="n">
         <v>-6973.532</v>
       </c>
-      <c r="Q6" s="20" t="n">
+      <c r="Q6" s="8" t="n">
         <v>-27192.559</v>
       </c>
-      <c r="R6" s="20" t="n">
+      <c r="R6" s="8" t="n">
         <v>-1077.38</v>
       </c>
-      <c r="S6" s="21" t="n">
+      <c r="S6" s="20" t="n">
         <v>352.478</v>
       </c>
-      <c r="T6" s="20" t="n">
+      <c r="T6" s="8" t="n">
         <v>-26027.013</v>
       </c>
-      <c r="U6" s="20" t="n">
+      <c r="U6" s="8" t="n">
         <v>-30488.34</v>
       </c>
-      <c r="V6" s="20" t="n">
+      <c r="V6" s="8" t="n">
         <v>-46838.632</v>
       </c>
-      <c r="W6" s="20" t="n">
+      <c r="W6" s="8" t="n">
         <v>-12809.786</v>
       </c>
-      <c r="X6" s="20" t="n">
+      <c r="X6" s="8" t="n">
         <v>-35033.5</v>
       </c>
-      <c r="Y6" s="20" t="n">
+      <c r="Y6" s="8" t="n">
         <v>-46541.023</v>
       </c>
-      <c r="Z6" s="21" t="n">
+      <c r="Z6" s="20" t="n">
         <v>233.715</v>
       </c>
-      <c r="AA6" s="20" t="n">
+      <c r="AA6" s="8" t="n">
         <v>-186347.058</v>
       </c>
-      <c r="AB6" s="20" t="n">
+      <c r="AB6" s="8" t="n">
         <v>-22296.357</v>
       </c>
-      <c r="AC6" s="21" t="n">
+      <c r="AC6" s="20" t="n">
         <v>11678.488</v>
       </c>
     </row>
@@ -4754,207 +4760,207 @@
       <c r="B7" s="19" t="n">
         <v>1809</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="20" t="n">
         <v>9094.619000000001</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="20" t="n">
         <v>1536.537</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="20" t="n">
         <v>15954.153</v>
       </c>
-      <c r="F7" s="21" t="n">
+      <c r="F7" s="20" t="n">
         <v>3231.403</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="20" t="n">
         <v>12183.568</v>
       </c>
-      <c r="H7" s="21" t="n">
+      <c r="H7" s="20" t="n">
         <v>9945.445</v>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="20" t="n">
         <v>13309.467</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="J7" s="20" t="n">
         <v>19229.181</v>
       </c>
-      <c r="K7" s="20" t="n">
+      <c r="K7" s="8" t="n">
         <v>-18947.937</v>
       </c>
-      <c r="L7" s="21" t="n">
+      <c r="L7" s="20" t="n">
         <v>19521.306</v>
       </c>
-      <c r="M7" s="21" t="n">
+      <c r="M7" s="20" t="n">
         <v>111543.835</v>
       </c>
-      <c r="N7" s="21" t="n">
+      <c r="N7" s="20" t="n">
         <v>44910.037</v>
       </c>
-      <c r="O7" s="21" t="n">
+      <c r="O7" s="20" t="n">
         <v>64648.943</v>
       </c>
-      <c r="P7" s="21" t="n">
+      <c r="P7" s="20" t="n">
         <v>88570.25199999999</v>
       </c>
-      <c r="Q7" s="21" t="n">
+      <c r="Q7" s="20" t="n">
         <v>43320.612</v>
       </c>
-      <c r="R7" s="20" t="n">
+      <c r="R7" s="8" t="n">
         <v>-18963.647</v>
       </c>
-      <c r="S7" s="21" t="n">
+      <c r="S7" s="20" t="n">
         <v>79414.034</v>
       </c>
-      <c r="T7" s="21" t="n">
+      <c r="T7" s="20" t="n">
         <v>45249.193</v>
       </c>
-      <c r="U7" s="21" t="n">
+      <c r="U7" s="20" t="n">
         <v>36530.769</v>
       </c>
-      <c r="V7" s="21" t="n">
+      <c r="V7" s="20" t="n">
         <v>127568.06</v>
       </c>
-      <c r="W7" s="20" t="n">
+      <c r="W7" s="8" t="n">
         <v>-19509.913</v>
       </c>
-      <c r="X7" s="21" t="n">
+      <c r="X7" s="20" t="n">
         <v>76002.281</v>
       </c>
-      <c r="Y7" s="21" t="n">
+      <c r="Y7" s="20" t="n">
         <v>139533.68</v>
       </c>
-      <c r="Z7" s="20" t="n">
+      <c r="Z7" s="8" t="n">
         <v>-18023.368</v>
       </c>
-      <c r="AA7" s="21" t="n">
+      <c r="AA7" s="20" t="n">
         <v>211370.114</v>
       </c>
-      <c r="AB7" s="21" t="n">
+      <c r="AB7" s="20" t="n">
         <v>73663.50999999999</v>
       </c>
-      <c r="AC7" s="20" t="n">
+      <c r="AC7" s="8" t="n">
         <v>-236.233</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">    Títulos — mercado primário</t>
         </is>
       </c>
-      <c r="B8" s="23" t="n">
+      <c r="B8" s="22" t="n">
         <v>29004</v>
       </c>
-      <c r="C8" s="24" t="n"/>
-      <c r="D8" s="24" t="n"/>
-      <c r="E8" s="24" t="n"/>
-      <c r="F8" s="24" t="n"/>
-      <c r="G8" s="24" t="n"/>
-      <c r="H8" s="24" t="n"/>
-      <c r="I8" s="24" t="n"/>
-      <c r="J8" s="24" t="n"/>
-      <c r="K8" s="24" t="n"/>
-      <c r="L8" s="24" t="n"/>
-      <c r="M8" s="24" t="n"/>
-      <c r="N8" s="24" t="n"/>
-      <c r="O8" s="24" t="n"/>
-      <c r="P8" s="24" t="n"/>
-      <c r="Q8" s="24" t="n"/>
-      <c r="R8" s="25" t="n">
+      <c r="C8" s="23" t="n"/>
+      <c r="D8" s="23" t="n"/>
+      <c r="E8" s="23" t="n"/>
+      <c r="F8" s="23" t="n"/>
+      <c r="G8" s="23" t="n"/>
+      <c r="H8" s="23" t="n"/>
+      <c r="I8" s="23" t="n"/>
+      <c r="J8" s="23" t="n"/>
+      <c r="K8" s="23" t="n"/>
+      <c r="L8" s="23" t="n"/>
+      <c r="M8" s="23" t="n"/>
+      <c r="N8" s="23" t="n"/>
+      <c r="O8" s="23" t="n"/>
+      <c r="P8" s="23" t="n"/>
+      <c r="Q8" s="23" t="n"/>
+      <c r="R8" s="8" t="n">
         <v>-41100.11</v>
       </c>
-      <c r="S8" s="26" t="n">
+      <c r="S8" s="24" t="n">
         <v>7559.278</v>
       </c>
-      <c r="T8" s="25" t="n">
+      <c r="T8" s="8" t="n">
         <v>-30684.804</v>
       </c>
-      <c r="U8" s="25" t="n">
+      <c r="U8" s="8" t="n">
         <v>-29615.079</v>
       </c>
-      <c r="V8" s="25" t="n">
+      <c r="V8" s="8" t="n">
         <v>-15623.582</v>
       </c>
-      <c r="W8" s="25" t="n">
+      <c r="W8" s="8" t="n">
         <v>-179441.373</v>
       </c>
-      <c r="X8" s="25" t="n">
+      <c r="X8" s="8" t="n">
         <v>-61753.191</v>
       </c>
-      <c r="Y8" s="25" t="n">
+      <c r="Y8" s="8" t="n">
         <v>-22231.419</v>
       </c>
-      <c r="Z8" s="25" t="n">
+      <c r="Z8" s="8" t="n">
         <v>-127402.891</v>
       </c>
-      <c r="AA8" s="25" t="n">
+      <c r="AA8" s="8" t="n">
         <v>-30736.668</v>
       </c>
-      <c r="AB8" s="25" t="n">
+      <c r="AB8" s="8" t="n">
         <v>-77293.57799999999</v>
       </c>
-      <c r="AC8" s="26" t="n">
+      <c r="AC8" s="24" t="n">
         <v>107193.514</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">    Títulos — mercado secundário</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n">
+      <c r="B9" s="22" t="n">
         <v>29006</v>
       </c>
-      <c r="C9" s="24" t="n"/>
-      <c r="D9" s="24" t="n"/>
-      <c r="E9" s="24" t="n"/>
-      <c r="F9" s="24" t="n"/>
-      <c r="G9" s="24" t="n"/>
-      <c r="H9" s="24" t="n"/>
-      <c r="I9" s="24" t="n"/>
-      <c r="J9" s="24" t="n"/>
-      <c r="K9" s="24" t="n"/>
-      <c r="L9" s="24" t="n"/>
-      <c r="M9" s="24" t="n"/>
-      <c r="N9" s="24" t="n"/>
-      <c r="O9" s="24" t="n"/>
-      <c r="P9" s="24" t="n"/>
-      <c r="Q9" s="24" t="n"/>
-      <c r="R9" s="26" t="n">
+      <c r="C9" s="23" t="n"/>
+      <c r="D9" s="23" t="n"/>
+      <c r="E9" s="23" t="n"/>
+      <c r="F9" s="23" t="n"/>
+      <c r="G9" s="23" t="n"/>
+      <c r="H9" s="23" t="n"/>
+      <c r="I9" s="23" t="n"/>
+      <c r="J9" s="23" t="n"/>
+      <c r="K9" s="23" t="n"/>
+      <c r="L9" s="23" t="n"/>
+      <c r="M9" s="23" t="n"/>
+      <c r="N9" s="23" t="n"/>
+      <c r="O9" s="23" t="n"/>
+      <c r="P9" s="23" t="n"/>
+      <c r="Q9" s="23" t="n"/>
+      <c r="R9" s="24" t="n">
         <v>22136.463</v>
       </c>
-      <c r="S9" s="26" t="n">
+      <c r="S9" s="24" t="n">
         <v>71854.75599999999</v>
       </c>
-      <c r="T9" s="26" t="n">
+      <c r="T9" s="24" t="n">
         <v>75933.997</v>
       </c>
-      <c r="U9" s="26" t="n">
+      <c r="U9" s="24" t="n">
         <v>66145.848</v>
       </c>
-      <c r="V9" s="26" t="n">
+      <c r="V9" s="24" t="n">
         <v>143191.642</v>
       </c>
-      <c r="W9" s="26" t="n">
+      <c r="W9" s="24" t="n">
         <v>159931.46</v>
       </c>
-      <c r="X9" s="26" t="n">
+      <c r="X9" s="24" t="n">
         <v>137755.472</v>
       </c>
-      <c r="Y9" s="26" t="n">
+      <c r="Y9" s="24" t="n">
         <v>161765.099</v>
       </c>
-      <c r="Z9" s="26" t="n">
+      <c r="Z9" s="24" t="n">
         <v>109379.523</v>
       </c>
-      <c r="AA9" s="26" t="n">
+      <c r="AA9" s="24" t="n">
         <v>242106.782</v>
       </c>
-      <c r="AB9" s="26" t="n">
+      <c r="AB9" s="24" t="n">
         <v>150957.088</v>
       </c>
-      <c r="AC9" s="25" t="n">
+      <c r="AC9" s="8" t="n">
         <v>-107429.747</v>
       </c>
     </row>
@@ -4967,85 +4973,85 @@
       <c r="B10" s="19" t="n">
         <v>1815</v>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="8" t="n">
         <v>-127.452</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="8" t="n">
         <v>-614.102</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="8" t="n">
         <v>-276.31</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="8" t="n">
         <v>-1665.84</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="8" t="n">
         <v>-1577.674</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="8" t="n">
         <v>-1927.55</v>
       </c>
-      <c r="I10" s="20" t="n">
+      <c r="I10" s="8" t="n">
         <v>-1645.963</v>
       </c>
-      <c r="J10" s="20" t="n">
+      <c r="J10" s="8" t="n">
         <v>-3466.24</v>
       </c>
-      <c r="K10" s="21" t="n">
+      <c r="K10" s="20" t="n">
         <v>44336.711</v>
       </c>
-      <c r="L10" s="20" t="n">
+      <c r="L10" s="8" t="n">
         <v>-2009.398</v>
       </c>
-      <c r="M10" s="20" t="n">
+      <c r="M10" s="8" t="n">
         <v>-65142.76</v>
       </c>
-      <c r="N10" s="21" t="n">
+      <c r="N10" s="20" t="n">
         <v>4361.607</v>
       </c>
-      <c r="O10" s="21" t="n">
+      <c r="O10" s="20" t="n">
         <v>3161.327</v>
       </c>
-      <c r="P10" s="20" t="n">
+      <c r="P10" s="8" t="n">
         <v>-7111.959</v>
       </c>
-      <c r="Q10" s="21" t="n">
+      <c r="Q10" s="20" t="n">
         <v>6483.102</v>
       </c>
-      <c r="R10" s="20" t="n">
+      <c r="R10" s="8" t="n">
         <v>-7713.625</v>
       </c>
-      <c r="S10" s="21" t="n">
+      <c r="S10" s="20" t="n">
         <v>1612.164</v>
       </c>
-      <c r="T10" s="21" t="n">
+      <c r="T10" s="20" t="n">
         <v>4770.938</v>
       </c>
-      <c r="U10" s="20" t="n">
+      <c r="U10" s="8" t="n">
         <v>-6759.022</v>
       </c>
-      <c r="V10" s="20" t="n">
+      <c r="V10" s="8" t="n">
         <v>-6659.602</v>
       </c>
-      <c r="W10" s="21" t="n">
+      <c r="W10" s="20" t="n">
         <v>3009.625</v>
       </c>
-      <c r="X10" s="21" t="n">
+      <c r="X10" s="20" t="n">
         <v>246.624</v>
       </c>
-      <c r="Y10" s="21" t="n">
+      <c r="Y10" s="20" t="n">
         <v>13351.98</v>
       </c>
-      <c r="Z10" s="20" t="n">
+      <c r="Z10" s="8" t="n">
         <v>-16363.195</v>
       </c>
-      <c r="AA10" s="21" t="n">
+      <c r="AA10" s="20" t="n">
         <v>35522.321</v>
       </c>
-      <c r="AB10" s="20" t="n">
+      <c r="AB10" s="8" t="n">
         <v>-20160.853</v>
       </c>
-      <c r="AC10" s="21" t="n">
+      <c r="AC10" s="20" t="n">
         <v>12119.269</v>
       </c>
     </row>
@@ -5058,81 +5064,81 @@
       <c r="B11" s="19" t="n">
         <v>12484</v>
       </c>
-      <c r="C11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="20" t="n">
+      <c r="C11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="8" t="n">
         <v>-0.9320000000000001</v>
       </c>
-      <c r="F11" s="20" t="n">
+      <c r="F11" s="8" t="n">
         <v>-3.965</v>
       </c>
-      <c r="G11" s="20" t="n">
+      <c r="G11" s="8" t="n">
         <v>-1.331</v>
       </c>
-      <c r="H11" s="20" t="n">
+      <c r="H11" s="8" t="n">
         <v>-0.102</v>
       </c>
-      <c r="I11" s="20" t="n">
+      <c r="I11" s="8" t="n">
         <v>-0.039</v>
       </c>
-      <c r="J11" s="20" t="n">
+      <c r="J11" s="8" t="n">
         <v>-0.05</v>
       </c>
-      <c r="K11" s="20" t="n">
+      <c r="K11" s="8" t="n">
         <v>-0.007</v>
       </c>
-      <c r="L11" s="20" t="n">
+      <c r="L11" s="8" t="n">
         <v>-0.031</v>
       </c>
-      <c r="M11" s="20" t="n">
+      <c r="M11" s="8" t="n">
         <v>-134.314</v>
       </c>
-      <c r="N11" s="20" t="n">
+      <c r="N11" s="8" t="n">
         <v>-0.001</v>
       </c>
-      <c r="O11" s="20" t="n">
+      <c r="O11" s="8" t="n">
         <v>-5.424</v>
       </c>
-      <c r="P11" s="20" t="n">
+      <c r="P11" s="8" t="n">
         <v>-0.002</v>
       </c>
-      <c r="Q11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="20" t="n">
+      <c r="Q11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="8" t="n">
         <v>-1.959</v>
       </c>
-      <c r="S11" s="20" t="n">
+      <c r="S11" s="8" t="n">
         <v>-0.027</v>
       </c>
-      <c r="T11" s="20" t="n">
+      <c r="T11" s="8" t="n">
         <v>-8.92</v>
       </c>
-      <c r="U11" s="21" t="n">
+      <c r="U11" s="20" t="n">
         <v>13.279</v>
       </c>
-      <c r="V11" s="20" t="n">
+      <c r="V11" s="8" t="n">
         <v>-0.06</v>
       </c>
-      <c r="W11" s="21" t="n">
+      <c r="W11" s="20" t="n">
         <v>2.383</v>
       </c>
-      <c r="X11" s="21" t="n">
+      <c r="X11" s="20" t="n">
         <v>50.194</v>
       </c>
-      <c r="Y11" s="21" t="n">
+      <c r="Y11" s="20" t="n">
         <v>26.424</v>
       </c>
-      <c r="Z11" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA11" s="27" t="n"/>
-      <c r="AB11" s="27" t="n"/>
-      <c r="AC11" s="27" t="n"/>
+      <c r="Z11" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="25" t="n"/>
+      <c r="AB11" s="25" t="n"/>
+      <c r="AC11" s="25" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -5143,81 +5149,81 @@
       <c r="B12" s="19" t="n">
         <v>12487</v>
       </c>
-      <c r="C12" s="27" t="n"/>
-      <c r="D12" s="27" t="n"/>
-      <c r="E12" s="21" t="n">
+      <c r="C12" s="25" t="n"/>
+      <c r="D12" s="25" t="n"/>
+      <c r="E12" s="20" t="n">
         <v>1707.304</v>
       </c>
-      <c r="F12" s="20" t="n">
+      <c r="F12" s="8" t="n">
         <v>-2507.953</v>
       </c>
-      <c r="G12" s="20" t="n">
+      <c r="G12" s="8" t="n">
         <v>-1581.56</v>
       </c>
-      <c r="H12" s="20" t="n">
+      <c r="H12" s="8" t="n">
         <v>-172.064</v>
       </c>
-      <c r="I12" s="21" t="n">
+      <c r="I12" s="20" t="n">
         <v>498.916</v>
       </c>
-      <c r="J12" s="21" t="n">
+      <c r="J12" s="20" t="n">
         <v>484.911</v>
       </c>
-      <c r="K12" s="21" t="n">
+      <c r="K12" s="20" t="n">
         <v>983.582</v>
       </c>
-      <c r="L12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="20" t="n">
+      <c r="L12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>-31.85</v>
       </c>
-      <c r="O12" s="20" t="n">
+      <c r="O12" s="8" t="n">
         <v>-59.77</v>
       </c>
-      <c r="P12" s="21" t="n">
+      <c r="P12" s="20" t="n">
         <v>48.593</v>
       </c>
-      <c r="Q12" s="21" t="n">
+      <c r="Q12" s="20" t="n">
         <v>17044.874</v>
       </c>
-      <c r="R12" s="21" t="n">
+      <c r="R12" s="20" t="n">
         <v>7794.459</v>
       </c>
-      <c r="S12" s="20" t="n">
+      <c r="S12" s="8" t="n">
         <v>-3858.12</v>
       </c>
-      <c r="T12" s="21" t="n">
+      <c r="T12" s="20" t="n">
         <v>1443.181</v>
       </c>
-      <c r="U12" s="21" t="n">
+      <c r="U12" s="20" t="n">
         <v>1519.905</v>
       </c>
-      <c r="V12" s="20" t="n">
+      <c r="V12" s="8" t="n">
         <v>-6928.091</v>
       </c>
-      <c r="W12" s="20" t="n">
+      <c r="W12" s="8" t="n">
         <v>-8028.787</v>
       </c>
-      <c r="X12" s="21" t="n">
+      <c r="X12" s="20" t="n">
         <v>3983.847</v>
       </c>
-      <c r="Y12" s="20" t="n">
+      <c r="Y12" s="8" t="n">
         <v>-5739.568</v>
       </c>
-      <c r="Z12" s="20" t="n">
+      <c r="Z12" s="8" t="n">
         <v>-6628.462</v>
       </c>
-      <c r="AA12" s="21" t="n">
+      <c r="AA12" s="20" t="n">
         <v>19928.148</v>
       </c>
-      <c r="AB12" s="21" t="n">
+      <c r="AB12" s="20" t="n">
         <v>18302.009</v>
       </c>
-      <c r="AC12" s="20" t="n">
+      <c r="AC12" s="8" t="n">
         <v>-12402.343</v>
       </c>
     </row>
@@ -5230,45 +5236,45 @@
       <c r="B13" s="19" t="n">
         <v>28724</v>
       </c>
-      <c r="C13" s="27" t="n"/>
-      <c r="D13" s="27" t="n"/>
-      <c r="E13" s="27" t="n"/>
-      <c r="F13" s="27" t="n"/>
-      <c r="G13" s="27" t="n"/>
-      <c r="H13" s="27" t="n"/>
-      <c r="I13" s="27" t="n"/>
-      <c r="J13" s="27" t="n"/>
-      <c r="K13" s="27" t="n"/>
-      <c r="L13" s="27" t="n"/>
-      <c r="M13" s="27" t="n"/>
-      <c r="N13" s="27" t="n"/>
-      <c r="O13" s="27" t="n"/>
-      <c r="P13" s="27" t="n"/>
-      <c r="Q13" s="27" t="n"/>
-      <c r="R13" s="27" t="n"/>
-      <c r="S13" s="27" t="n"/>
-      <c r="T13" s="27" t="n"/>
-      <c r="U13" s="27" t="n"/>
-      <c r="V13" s="27" t="n"/>
-      <c r="W13" s="21" t="n">
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="25" t="n"/>
+      <c r="I13" s="25" t="n"/>
+      <c r="J13" s="25" t="n"/>
+      <c r="K13" s="25" t="n"/>
+      <c r="L13" s="25" t="n"/>
+      <c r="M13" s="25" t="n"/>
+      <c r="N13" s="25" t="n"/>
+      <c r="O13" s="25" t="n"/>
+      <c r="P13" s="25" t="n"/>
+      <c r="Q13" s="25" t="n"/>
+      <c r="R13" s="25" t="n"/>
+      <c r="S13" s="25" t="n"/>
+      <c r="T13" s="25" t="n"/>
+      <c r="U13" s="25" t="n"/>
+      <c r="V13" s="25" t="n"/>
+      <c r="W13" s="20" t="n">
         <v>27816.1</v>
       </c>
-      <c r="X13" s="21" t="n">
+      <c r="X13" s="20" t="n">
         <v>4765.473</v>
       </c>
-      <c r="Y13" s="20" t="n">
+      <c r="Y13" s="8" t="n">
         <v>-17642.115</v>
       </c>
-      <c r="Z13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB13" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC13" s="20" t="n">
+      <c r="Z13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="8" t="n">
         <v>-805.306</v>
       </c>
     </row>
@@ -5281,85 +5287,85 @@
       <c r="B14" s="19" t="n">
         <v>1818</v>
       </c>
-      <c r="C14" s="21" t="n">
+      <c r="C14" s="20" t="n">
         <v>20.253</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="8" t="n">
         <v>-66.297</v>
       </c>
-      <c r="E14" s="21" t="n">
+      <c r="E14" s="20" t="n">
         <v>143.984</v>
       </c>
-      <c r="F14" s="21" t="n">
+      <c r="F14" s="20" t="n">
         <v>22.977</v>
       </c>
-      <c r="G14" s="21" t="n">
+      <c r="G14" s="20" t="n">
         <v>214.898</v>
       </c>
-      <c r="H14" s="21" t="n">
+      <c r="H14" s="20" t="n">
         <v>144.777</v>
       </c>
-      <c r="I14" s="21" t="n">
+      <c r="I14" s="20" t="n">
         <v>195.164</v>
       </c>
-      <c r="J14" s="21" t="n">
+      <c r="J14" s="20" t="n">
         <v>137.516</v>
       </c>
-      <c r="K14" s="21" t="n">
+      <c r="K14" s="20" t="n">
         <v>182.436</v>
       </c>
-      <c r="L14" s="21" t="n">
+      <c r="L14" s="20" t="n">
         <v>541.211</v>
       </c>
-      <c r="M14" s="21" t="n">
+      <c r="M14" s="20" t="n">
         <v>704.9690000000001</v>
       </c>
-      <c r="N14" s="20" t="n">
+      <c r="N14" s="8" t="n">
         <v>-33.262</v>
       </c>
-      <c r="O14" s="21" t="n">
+      <c r="O14" s="20" t="n">
         <v>6957.731</v>
       </c>
-      <c r="P14" s="21" t="n">
+      <c r="P14" s="20" t="n">
         <v>2528.586</v>
       </c>
-      <c r="Q14" s="21" t="n">
+      <c r="Q14" s="20" t="n">
         <v>185.497</v>
       </c>
-      <c r="R14" s="21" t="n">
+      <c r="R14" s="20" t="n">
         <v>437.373</v>
       </c>
-      <c r="S14" s="21" t="n">
+      <c r="S14" s="20" t="n">
         <v>244.327</v>
       </c>
-      <c r="T14" s="20" t="n">
+      <c r="T14" s="8" t="n">
         <v>-55.314</v>
       </c>
-      <c r="U14" s="21" t="n">
+      <c r="U14" s="20" t="n">
         <v>1520.697</v>
       </c>
-      <c r="V14" s="20" t="n">
+      <c r="V14" s="8" t="n">
         <v>-3362.213</v>
       </c>
-      <c r="W14" s="20" t="n">
+      <c r="W14" s="8" t="n">
         <v>-1835.66</v>
       </c>
-      <c r="X14" s="20" t="n">
+      <c r="X14" s="8" t="n">
         <v>-11219.235</v>
       </c>
-      <c r="Y14" s="20" t="n">
+      <c r="Y14" s="8" t="n">
         <v>-19082.092</v>
       </c>
-      <c r="Z14" s="20" t="n">
+      <c r="Z14" s="8" t="n">
         <v>-22381.99</v>
       </c>
-      <c r="AA14" s="20" t="n">
+      <c r="AA14" s="8" t="n">
         <v>-10450.304</v>
       </c>
-      <c r="AB14" s="21" t="n">
+      <c r="AB14" s="20" t="n">
         <v>2448.268</v>
       </c>
-      <c r="AC14" s="20" t="n">
+      <c r="AC14" s="8" t="n">
         <v>-52006.568</v>
       </c>
     </row>
@@ -5372,85 +5378,85 @@
       <c r="B15" s="34" t="n">
         <v>1788</v>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="11" t="n">
         <v>47686.213</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="11" t="n">
         <v>53255.971</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="11" t="n">
         <v>73302.272</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="11" t="n">
         <v>73219.136</v>
       </c>
-      <c r="G15" s="12" t="n">
+      <c r="G15" s="11" t="n">
         <v>88732.677</v>
       </c>
-      <c r="H15" s="12" t="n">
+      <c r="H15" s="11" t="n">
         <v>101247.235</v>
       </c>
-      <c r="I15" s="12" t="n">
+      <c r="I15" s="11" t="n">
         <v>121102.001</v>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="11" t="n">
         <v>146616.867</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="K15" s="11" t="n">
         <v>147549.705</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="L15" s="11" t="n">
         <v>166072.835</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="M15" s="11" t="n">
         <v>206853.322</v>
       </c>
-      <c r="N15" s="12" t="n">
+      <c r="N15" s="11" t="n">
         <v>214235.311</v>
       </c>
-      <c r="O15" s="12" t="n">
+      <c r="O15" s="11" t="n">
         <v>233371.452</v>
       </c>
-      <c r="P15" s="12" t="n">
+      <c r="P15" s="11" t="n">
         <v>249509.778</v>
       </c>
-      <c r="Q15" s="12" t="n">
+      <c r="Q15" s="11" t="n">
         <v>263528.517</v>
       </c>
-      <c r="R15" s="12" t="n">
+      <c r="R15" s="11" t="n">
         <v>255288.922</v>
       </c>
-      <c r="S15" s="12" t="n">
+      <c r="S15" s="11" t="n">
         <v>270287.146</v>
       </c>
-      <c r="T15" s="12" t="n">
+      <c r="T15" s="11" t="n">
         <v>296755.456</v>
       </c>
-      <c r="U15" s="12" t="n">
+      <c r="U15" s="11" t="n">
         <v>302049.461</v>
       </c>
-      <c r="V15" s="12" t="n">
+      <c r="V15" s="11" t="n">
         <v>316586.707</v>
       </c>
-      <c r="W15" s="12" t="n">
+      <c r="W15" s="11" t="n">
         <v>431536.653</v>
       </c>
-      <c r="X15" s="12" t="n">
+      <c r="X15" s="11" t="n">
         <v>409183.519</v>
       </c>
-      <c r="Y15" s="12" t="n">
+      <c r="Y15" s="11" t="n">
         <v>419659.918</v>
       </c>
-      <c r="Z15" s="12" t="n">
+      <c r="Z15" s="11" t="n">
         <v>422718.628</v>
       </c>
-      <c r="AA15" s="12" t="n">
+      <c r="AA15" s="11" t="n">
         <v>451213.588</v>
       </c>
-      <c r="AB15" s="12" t="n">
+      <c r="AB15" s="11" t="n">
         <v>447096.654</v>
       </c>
-      <c r="AC15" s="12" t="n">
+      <c r="AC15" s="11" t="n">
         <v>432551.687</v>
       </c>
     </row>
@@ -5463,85 +5469,85 @@
       <c r="B16" s="19" t="n">
         <v>1786</v>
       </c>
-      <c r="C16" s="27" t="n">
+      <c r="C16" s="25" t="n">
         <v>32633.056</v>
       </c>
-      <c r="D16" s="27" t="n">
+      <c r="D16" s="25" t="n">
         <v>37668.836</v>
       </c>
-      <c r="E16" s="27" t="n">
+      <c r="E16" s="25" t="n">
         <v>49931.066</v>
       </c>
-      <c r="F16" s="27" t="n">
+      <c r="F16" s="25" t="n">
         <v>51363.863</v>
       </c>
-      <c r="G16" s="27" t="n">
+      <c r="G16" s="25" t="n">
         <v>61935.635</v>
       </c>
-      <c r="H16" s="27" t="n">
+      <c r="H16" s="25" t="n">
         <v>70033.641</v>
       </c>
-      <c r="I16" s="27" t="n">
+      <c r="I16" s="25" t="n">
         <v>85824.753</v>
       </c>
-      <c r="J16" s="27" t="n">
+      <c r="J16" s="25" t="n">
         <v>102885.047</v>
       </c>
-      <c r="K16" s="27" t="n">
+      <c r="K16" s="25" t="n">
         <v>115590.704</v>
       </c>
-      <c r="L16" s="27" t="n">
+      <c r="L16" s="25" t="n">
         <v>131861.185</v>
       </c>
-      <c r="M16" s="27" t="n">
+      <c r="M16" s="25" t="n">
         <v>151145.368</v>
       </c>
-      <c r="N16" s="27" t="n">
+      <c r="N16" s="25" t="n">
         <v>162769.67</v>
       </c>
-      <c r="O16" s="27" t="n">
+      <c r="O16" s="25" t="n">
         <v>187434.736</v>
       </c>
-      <c r="P16" s="27" t="n">
+      <c r="P16" s="25" t="n">
         <v>204052.42</v>
       </c>
-      <c r="Q16" s="27" t="n">
+      <c r="Q16" s="25" t="n">
         <v>220853.706</v>
       </c>
-      <c r="R16" s="27" t="n">
+      <c r="R16" s="25" t="n">
         <v>225485.184</v>
       </c>
-      <c r="S16" s="27" t="n">
+      <c r="S16" s="25" t="n">
         <v>232145.593</v>
       </c>
-      <c r="T16" s="27" t="n">
+      <c r="T16" s="25" t="n">
         <v>250363.681</v>
       </c>
-      <c r="U16" s="27" t="n">
+      <c r="U16" s="25" t="n">
         <v>264967.669</v>
       </c>
-      <c r="V16" s="27" t="n">
+      <c r="V16" s="25" t="n">
         <v>280685.185</v>
       </c>
-      <c r="W16" s="27" t="n">
+      <c r="W16" s="25" t="n">
         <v>370441.036</v>
       </c>
-      <c r="X16" s="27" t="n">
+      <c r="X16" s="25" t="n">
         <v>339013.043</v>
       </c>
-      <c r="Y16" s="27" t="n">
+      <c r="Y16" s="25" t="n">
         <v>342334.138</v>
       </c>
-      <c r="Z16" s="27" t="n">
+      <c r="Z16" s="25" t="n">
         <v>341616.828</v>
       </c>
-      <c r="AA16" s="27" t="n">
+      <c r="AA16" s="25" t="n">
         <v>355858.101</v>
       </c>
-      <c r="AB16" s="27" t="n">
+      <c r="AB16" s="25" t="n">
         <v>368625.466</v>
       </c>
-      <c r="AC16" s="27" t="n">
+      <c r="AC16" s="25" t="n">
         <v>382994.849</v>
       </c>
     </row>
@@ -5554,85 +5560,85 @@
       <c r="B17" s="19" t="n">
         <v>1787</v>
       </c>
-      <c r="C17" s="27" t="n">
+      <c r="C17" s="25" t="n">
         <v>15053.157</v>
       </c>
-      <c r="D17" s="27" t="n">
+      <c r="D17" s="25" t="n">
         <v>15587.135</v>
       </c>
-      <c r="E17" s="27" t="n">
+      <c r="E17" s="25" t="n">
         <v>23371.206</v>
       </c>
-      <c r="F17" s="27" t="n">
+      <c r="F17" s="25" t="n">
         <v>21855.273</v>
       </c>
-      <c r="G17" s="27" t="n">
+      <c r="G17" s="25" t="n">
         <v>26797.042</v>
       </c>
-      <c r="H17" s="27" t="n">
+      <c r="H17" s="25" t="n">
         <v>31213.594</v>
       </c>
-      <c r="I17" s="27" t="n">
+      <c r="I17" s="25" t="n">
         <v>35277.248</v>
       </c>
-      <c r="J17" s="27" t="n">
+      <c r="J17" s="25" t="n">
         <v>43731.82</v>
       </c>
-      <c r="K17" s="27" t="n">
+      <c r="K17" s="25" t="n">
         <v>31959.001</v>
       </c>
-      <c r="L17" s="27" t="n">
+      <c r="L17" s="25" t="n">
         <v>34211.65</v>
       </c>
-      <c r="M17" s="27" t="n">
+      <c r="M17" s="25" t="n">
         <v>55707.954</v>
       </c>
-      <c r="N17" s="27" t="n">
+      <c r="N17" s="25" t="n">
         <v>51465.641</v>
       </c>
-      <c r="O17" s="27" t="n">
+      <c r="O17" s="25" t="n">
         <v>45936.716</v>
       </c>
-      <c r="P17" s="27" t="n">
+      <c r="P17" s="25" t="n">
         <v>45457.358</v>
       </c>
-      <c r="Q17" s="27" t="n">
+      <c r="Q17" s="25" t="n">
         <v>42674.811</v>
       </c>
-      <c r="R17" s="27" t="n">
+      <c r="R17" s="25" t="n">
         <v>29803.738</v>
       </c>
-      <c r="S17" s="27" t="n">
+      <c r="S17" s="25" t="n">
         <v>38141.553</v>
       </c>
-      <c r="T17" s="27" t="n">
+      <c r="T17" s="25" t="n">
         <v>46391.775</v>
       </c>
-      <c r="U17" s="27" t="n">
+      <c r="U17" s="25" t="n">
         <v>37081.792</v>
       </c>
-      <c r="V17" s="27" t="n">
+      <c r="V17" s="25" t="n">
         <v>35901.522</v>
       </c>
-      <c r="W17" s="27" t="n">
+      <c r="W17" s="25" t="n">
         <v>61095.617</v>
       </c>
-      <c r="X17" s="27" t="n">
+      <c r="X17" s="25" t="n">
         <v>70170.476</v>
       </c>
-      <c r="Y17" s="27" t="n">
+      <c r="Y17" s="25" t="n">
         <v>77325.78</v>
       </c>
-      <c r="Z17" s="27" t="n">
+      <c r="Z17" s="25" t="n">
         <v>81101.8</v>
       </c>
-      <c r="AA17" s="27" t="n">
+      <c r="AA17" s="25" t="n">
         <v>95355.488</v>
       </c>
-      <c r="AB17" s="27" t="n">
+      <c r="AB17" s="25" t="n">
         <v>78471.18799999999</v>
       </c>
-      <c r="AC17" s="27" t="n">
+      <c r="AC17" s="25" t="n">
         <v>49556.839</v>
       </c>
     </row>

</xml_diff>